<commit_message>
chore(data): refresh deployed fixtures to the current generation
The deployed workbooks were stale: they were generated when the county pool was
intersected with the local 302-county sample, whereas the fixtures now draw from
the full national warehouse pool. 299 of 300 rows differ (row 1 moved CA -> AK).

- Re-copy all 8 .xlsx + 8 expectations .csv from backend/fixtures.
- Migration refreshes sampleRows so the on-page table matches the downloadable
  file — otherwise the page shows one dataset and the download contains another.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53946,7 +53946,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>90265</t>
+          <t>94501</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -54215,7 +54215,7 @@
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>10463</t>
+          <t>12009</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
@@ -54484,7 +54484,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>60007</t>
+          <t>62311</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -54769,7 +54769,7 @@
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>90265</t>
+          <t>94501</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
@@ -55038,7 +55038,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>90265</t>
+          <t>94501</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -55303,7 +55303,7 @@
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>77031</t>
+          <t>75751</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
@@ -55837,7 +55837,7 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>10463</t>
+          <t>12009</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
@@ -56375,7 +56375,7 @@
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>77031</t>
+          <t>75751</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
@@ -56644,7 +56644,7 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>60007</t>
+          <t>62311</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
@@ -56913,7 +56913,7 @@
       </c>
       <c r="E29" s="14" t="inlineStr">
         <is>
-          <t>60007</t>
+          <t>62311</t>
         </is>
       </c>
       <c r="F29" s="14" t="inlineStr">
@@ -57182,7 +57182,7 @@
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>77031</t>
+          <t>75751</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
@@ -57451,7 +57451,7 @@
       </c>
       <c r="E31" s="14" t="inlineStr">
         <is>
-          <t>98022</t>
+          <t>98832</t>
         </is>
       </c>
       <c r="F31" s="14" t="inlineStr">
@@ -57720,7 +57720,7 @@
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>90265</t>
+          <t>94501</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
@@ -57989,7 +57989,7 @@
       </c>
       <c r="E33" s="14" t="inlineStr">
         <is>
-          <t>53507</t>
+          <t>53920</t>
         </is>
       </c>
       <c r="F33" s="14" t="inlineStr">
@@ -58258,7 +58258,7 @@
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>10463</t>
+          <t>12009</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
@@ -58527,7 +58527,7 @@
       </c>
       <c r="E35" s="14" t="inlineStr">
         <is>
-          <t>77031</t>
+          <t>75751</t>
         </is>
       </c>
       <c r="F35" s="14" t="inlineStr">

</xml_diff>

<commit_message>
fix(data): three census-realism bugs visible in the sample rows
Reviewing the deployed sample table surfaced three defects in the generated data:

1. Comp history ran BACKWARDS — 2025 total exceeded 2026 (a pay cut forward in
   time) because the base was stepped down 3%/yr and then a bonus added on top.
   Now the TOTAL steps down and base/bonus are derived from it: 0/300 rows
   non-monotonic (was 300/300).
2. Part-time employees showed 2,080 hours in prior years; hours now follow the
   row's actual schedule across all four years.
3. Every one of the 300 employees shared one DOB (05/10/1990), hire date
   (03/02/2020) and gender. Now 251 distinct DOBs, 212 hire dates, both genders.

Refreshes the downloadable workbooks and the on-page sample rows together.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53931,12 +53931,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>10/22/1991</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53976,7 +53976,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>04/08/2022</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54004,12 +54004,12 @@
       <c r="R18" s="14" t="n"/>
       <c r="S18" s="14" t="inlineStr">
         <is>
-          <t>$19.71</t>
+          <t>$18.94</t>
         </is>
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>$29.57</t>
+          <t>$28.41</t>
         </is>
       </c>
       <c r="U18" s="11" t="inlineStr">
@@ -54045,12 +54045,12 @@
       <c r="AA18" s="11" t="n"/>
       <c r="AB18" s="11" t="inlineStr">
         <is>
-          <t>$19.13</t>
+          <t>$18.37</t>
         </is>
       </c>
       <c r="AC18" s="11" t="inlineStr">
         <is>
-          <t>$28.70</t>
+          <t>$27.55</t>
         </is>
       </c>
       <c r="AD18" s="11" t="inlineStr">
@@ -54070,18 +54070,18 @@
       </c>
       <c r="AG18" s="11" t="inlineStr">
         <is>
-          <t>$41,400.00</t>
+          <t>$39,800.00</t>
         </is>
       </c>
       <c r="AH18" s="11" t="n"/>
       <c r="AI18" s="11" t="inlineStr">
         <is>
-          <t>$18.56</t>
+          <t>$17.84</t>
         </is>
       </c>
       <c r="AJ18" s="11" t="inlineStr">
         <is>
-          <t>$27.84</t>
+          <t>$26.76</t>
         </is>
       </c>
       <c r="AK18" s="11" t="inlineStr">
@@ -54101,18 +54101,18 @@
       </c>
       <c r="AN18" s="11" t="inlineStr">
         <is>
-          <t>$40,100.00</t>
+          <t>$38,600.00</t>
         </is>
       </c>
       <c r="AO18" s="11" t="n"/>
       <c r="AP18" s="11" t="inlineStr">
         <is>
-          <t>$18.03</t>
+          <t>$17.31</t>
         </is>
       </c>
       <c r="AQ18" s="11" t="inlineStr">
         <is>
-          <t>$27.05</t>
+          <t>$25.96</t>
         </is>
       </c>
       <c r="AR18" s="11" t="inlineStr">
@@ -54132,7 +54132,7 @@
       </c>
       <c r="AU18" s="11" t="inlineStr">
         <is>
-          <t>$39,000.00</t>
+          <t>$37,500.00</t>
         </is>
       </c>
       <c r="AV18" s="11" t="inlineStr">
@@ -54200,7 +54200,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>09/05/1962</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -54245,7 +54245,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>05/11/2023</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54273,12 +54273,12 @@
       <c r="R19" s="14" t="n"/>
       <c r="S19" s="14" t="inlineStr">
         <is>
-          <t>$19.71</t>
+          <t>$18.94</t>
         </is>
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>$29.57</t>
+          <t>$28.41</t>
         </is>
       </c>
       <c r="U19" s="11" t="inlineStr">
@@ -54314,12 +54314,12 @@
       <c r="AA19" s="11" t="n"/>
       <c r="AB19" s="11" t="inlineStr">
         <is>
-          <t>$19.13</t>
+          <t>$18.37</t>
         </is>
       </c>
       <c r="AC19" s="11" t="inlineStr">
         <is>
-          <t>$28.70</t>
+          <t>$27.55</t>
         </is>
       </c>
       <c r="AD19" s="11" t="inlineStr">
@@ -54339,18 +54339,18 @@
       </c>
       <c r="AG19" s="11" t="inlineStr">
         <is>
-          <t>$41,400.00</t>
+          <t>$39,800.00</t>
         </is>
       </c>
       <c r="AH19" s="11" t="n"/>
       <c r="AI19" s="11" t="inlineStr">
         <is>
-          <t>$18.56</t>
+          <t>$17.84</t>
         </is>
       </c>
       <c r="AJ19" s="11" t="inlineStr">
         <is>
-          <t>$27.84</t>
+          <t>$26.76</t>
         </is>
       </c>
       <c r="AK19" s="11" t="inlineStr">
@@ -54370,18 +54370,18 @@
       </c>
       <c r="AN19" s="11" t="inlineStr">
         <is>
-          <t>$40,100.00</t>
+          <t>$38,600.00</t>
         </is>
       </c>
       <c r="AO19" s="11" t="n"/>
       <c r="AP19" s="11" t="inlineStr">
         <is>
-          <t>$18.03</t>
+          <t>$17.31</t>
         </is>
       </c>
       <c r="AQ19" s="11" t="inlineStr">
         <is>
-          <t>$27.05</t>
+          <t>$25.96</t>
         </is>
       </c>
       <c r="AR19" s="11" t="inlineStr">
@@ -54401,7 +54401,7 @@
       </c>
       <c r="AU19" s="11" t="inlineStr">
         <is>
-          <t>$39,000.00</t>
+          <t>$37,500.00</t>
         </is>
       </c>
       <c r="AV19" s="11" t="inlineStr">
@@ -54469,7 +54469,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>05/05/1982</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -54514,7 +54514,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>01/02/2020</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54546,12 +54546,12 @@
       </c>
       <c r="S20" s="14" t="inlineStr">
         <is>
-          <t>$35.62</t>
+          <t>$34.18</t>
         </is>
       </c>
       <c r="T20" s="13" t="inlineStr">
         <is>
-          <t>$53.43</t>
+          <t>$51.27</t>
         </is>
       </c>
       <c r="U20" s="11" t="inlineStr">
@@ -54591,12 +54591,12 @@
       </c>
       <c r="AB20" s="11" t="inlineStr">
         <is>
-          <t>$34.57</t>
+          <t>$33.17</t>
         </is>
       </c>
       <c r="AC20" s="11" t="inlineStr">
         <is>
-          <t>$51.86</t>
+          <t>$49.76</t>
         </is>
       </c>
       <c r="AD20" s="11" t="inlineStr">
@@ -54626,12 +54626,12 @@
       </c>
       <c r="AI20" s="11" t="inlineStr">
         <is>
-          <t>$33.56</t>
+          <t>$32.21</t>
         </is>
       </c>
       <c r="AJ20" s="11" t="inlineStr">
         <is>
-          <t>$50.34</t>
+          <t>$48.31</t>
         </is>
       </c>
       <c r="AK20" s="11" t="inlineStr">
@@ -54661,12 +54661,12 @@
       </c>
       <c r="AP20" s="11" t="inlineStr">
         <is>
-          <t>$32.60</t>
+          <t>$31.30</t>
         </is>
       </c>
       <c r="AQ20" s="11" t="inlineStr">
         <is>
-          <t>$48.90</t>
+          <t>$46.95</t>
         </is>
       </c>
       <c r="AR20" s="11" t="inlineStr">
@@ -54754,7 +54754,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>09/05/1970</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
@@ -54799,7 +54799,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>05/11/2019</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -54827,12 +54827,12 @@
       <c r="R21" s="14" t="n"/>
       <c r="S21" s="14" t="inlineStr">
         <is>
-          <t>$20.14</t>
+          <t>$19.33</t>
         </is>
       </c>
       <c r="T21" s="13" t="inlineStr">
         <is>
-          <t>$30.21</t>
+          <t>$28.99</t>
         </is>
       </c>
       <c r="U21" s="11" t="inlineStr">
@@ -54868,12 +54868,12 @@
       <c r="AA21" s="11" t="n"/>
       <c r="AB21" s="11" t="inlineStr">
         <is>
-          <t>$19.57</t>
+          <t>$18.80</t>
         </is>
       </c>
       <c r="AC21" s="11" t="inlineStr">
         <is>
-          <t>$29.36</t>
+          <t>$28.20</t>
         </is>
       </c>
       <c r="AD21" s="11" t="inlineStr">
@@ -54893,18 +54893,18 @@
       </c>
       <c r="AG21" s="11" t="inlineStr">
         <is>
-          <t>$42,300.00</t>
+          <t>$40,700.00</t>
         </is>
       </c>
       <c r="AH21" s="11" t="n"/>
       <c r="AI21" s="11" t="inlineStr">
         <is>
-          <t>$18.99</t>
+          <t>$18.22</t>
         </is>
       </c>
       <c r="AJ21" s="11" t="inlineStr">
         <is>
-          <t>$28.48</t>
+          <t>$27.33</t>
         </is>
       </c>
       <c r="AK21" s="11" t="inlineStr">
@@ -54924,18 +54924,18 @@
       </c>
       <c r="AN21" s="11" t="inlineStr">
         <is>
-          <t>$41,100.00</t>
+          <t>$39,500.00</t>
         </is>
       </c>
       <c r="AO21" s="11" t="n"/>
       <c r="AP21" s="11" t="inlineStr">
         <is>
-          <t>$18.41</t>
+          <t>$17.69</t>
         </is>
       </c>
       <c r="AQ21" s="11" t="inlineStr">
         <is>
-          <t>$27.62</t>
+          <t>$26.54</t>
         </is>
       </c>
       <c r="AR21" s="11" t="inlineStr">
@@ -54955,7 +54955,7 @@
       </c>
       <c r="AU21" s="11" t="inlineStr">
         <is>
-          <t>$39,800.00</t>
+          <t>$38,300.00</t>
         </is>
       </c>
       <c r="AV21" s="11" t="inlineStr">
@@ -55023,7 +55023,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>09/13/1986</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -55068,7 +55068,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>10/23/2013</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55096,12 +55096,12 @@
       <c r="R22" s="14" t="n"/>
       <c r="S22" s="14" t="inlineStr">
         <is>
-          <t>$15.38</t>
+          <t>$14.76</t>
         </is>
       </c>
       <c r="T22" s="13" t="inlineStr">
         <is>
-          <t>$23.07</t>
+          <t>$22.14</t>
         </is>
       </c>
       <c r="U22" s="11" t="inlineStr">
@@ -55137,12 +55137,12 @@
       <c r="AA22" s="11" t="n"/>
       <c r="AB22" s="11" t="inlineStr">
         <is>
-          <t>$14.95</t>
+          <t>$14.38</t>
         </is>
       </c>
       <c r="AC22" s="11" t="inlineStr">
         <is>
-          <t>$22.42</t>
+          <t>$21.57</t>
         </is>
       </c>
       <c r="AD22" s="11" t="inlineStr">
@@ -55162,18 +55162,18 @@
       </c>
       <c r="AG22" s="11" t="inlineStr">
         <is>
-          <t>$32,300.00</t>
+          <t>$31,100.00</t>
         </is>
       </c>
       <c r="AH22" s="11" t="n"/>
       <c r="AI22" s="11" t="inlineStr">
         <is>
-          <t>$14.52</t>
+          <t>$13.94</t>
         </is>
       </c>
       <c r="AJ22" s="11" t="inlineStr">
         <is>
-          <t>$21.78</t>
+          <t>$20.91</t>
         </is>
       </c>
       <c r="AK22" s="11" t="inlineStr">
@@ -55193,18 +55193,18 @@
       </c>
       <c r="AN22" s="11" t="inlineStr">
         <is>
-          <t>$31,400.00</t>
+          <t>$30,200.00</t>
         </is>
       </c>
       <c r="AO22" s="11" t="n"/>
       <c r="AP22" s="11" t="inlineStr">
         <is>
-          <t>$14.09</t>
+          <t>$13.51</t>
         </is>
       </c>
       <c r="AQ22" s="11" t="inlineStr">
         <is>
-          <t>$21.13</t>
+          <t>$20.27</t>
         </is>
       </c>
       <c r="AR22" s="11" t="inlineStr">
@@ -55224,7 +55224,7 @@
       </c>
       <c r="AU22" s="11" t="inlineStr">
         <is>
-          <t>$30,500.00</t>
+          <t>$29,300.00</t>
         </is>
       </c>
       <c r="AV22" s="11" t="inlineStr">
@@ -55288,7 +55288,7 @@
       <c r="A23" s="23" t="inlineStr"/>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>01/01/1962</t>
         </is>
       </c>
       <c r="C23" s="21" t="inlineStr">
@@ -55333,7 +55333,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>01/01/2012</t>
         </is>
       </c>
       <c r="L23" s="14" t="n"/>
@@ -55361,12 +55361,12 @@
       <c r="R23" s="14" t="n"/>
       <c r="S23" s="14" t="inlineStr">
         <is>
-          <t>$16.44</t>
+          <t>$15.77</t>
         </is>
       </c>
       <c r="T23" s="13" t="inlineStr">
         <is>
-          <t>$24.66</t>
+          <t>$23.66</t>
         </is>
       </c>
       <c r="U23" s="11" t="inlineStr">
@@ -55402,12 +55402,12 @@
       <c r="AA23" s="11" t="n"/>
       <c r="AB23" s="11" t="inlineStr">
         <is>
-          <t>$15.96</t>
+          <t>$15.34</t>
         </is>
       </c>
       <c r="AC23" s="11" t="inlineStr">
         <is>
-          <t>$23.94</t>
+          <t>$23.01</t>
         </is>
       </c>
       <c r="AD23" s="11" t="inlineStr">
@@ -55427,18 +55427,18 @@
       </c>
       <c r="AG23" s="11" t="inlineStr">
         <is>
-          <t>$34,500.00</t>
+          <t>$33,200.00</t>
         </is>
       </c>
       <c r="AH23" s="11" t="n"/>
       <c r="AI23" s="11" t="inlineStr">
         <is>
-          <t>$15.48</t>
+          <t>$14.86</t>
         </is>
       </c>
       <c r="AJ23" s="11" t="inlineStr">
         <is>
-          <t>$23.22</t>
+          <t>$22.29</t>
         </is>
       </c>
       <c r="AK23" s="11" t="inlineStr">
@@ -55458,18 +55458,18 @@
       </c>
       <c r="AN23" s="11" t="inlineStr">
         <is>
-          <t>$33,500.00</t>
+          <t>$32,200.00</t>
         </is>
       </c>
       <c r="AO23" s="11" t="n"/>
       <c r="AP23" s="11" t="inlineStr">
         <is>
-          <t>$15.05</t>
+          <t>$14.42</t>
         </is>
       </c>
       <c r="AQ23" s="11" t="inlineStr">
         <is>
-          <t>$22.58</t>
+          <t>$21.63</t>
         </is>
       </c>
       <c r="AR23" s="11" t="inlineStr">
@@ -55489,7 +55489,7 @@
       </c>
       <c r="AU23" s="11" t="inlineStr">
         <is>
-          <t>$32,600.00</t>
+          <t>$31,300.00</t>
         </is>
       </c>
       <c r="AV23" s="11" t="inlineStr">
@@ -55557,7 +55557,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>09/05/1994</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -55598,7 +55598,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>05/11/2018</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55626,12 +55626,12 @@
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="inlineStr">
         <is>
-          <t>$33.70</t>
+          <t>$32.36</t>
         </is>
       </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
-          <t>$50.55</t>
+          <t>$48.54</t>
         </is>
       </c>
       <c r="U24" s="11" t="inlineStr">
@@ -55667,12 +55667,12 @@
       <c r="AA24" s="11" t="n"/>
       <c r="AB24" s="11" t="inlineStr">
         <is>
-          <t>$32.74</t>
+          <t>$31.44</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>$49.11</t>
+          <t>$47.16</t>
         </is>
       </c>
       <c r="AD24" s="11" t="inlineStr">
@@ -55692,18 +55692,18 @@
       </c>
       <c r="AG24" s="11" t="inlineStr">
         <is>
-          <t>$70,800.00</t>
+          <t>$68,100.00</t>
         </is>
       </c>
       <c r="AH24" s="11" t="n"/>
       <c r="AI24" s="11" t="inlineStr">
         <is>
-          <t>$31.78</t>
+          <t>$30.53</t>
         </is>
       </c>
       <c r="AJ24" s="11" t="inlineStr">
         <is>
-          <t>$47.67</t>
+          <t>$45.80</t>
         </is>
       </c>
       <c r="AK24" s="11" t="inlineStr">
@@ -55723,18 +55723,18 @@
       </c>
       <c r="AN24" s="11" t="inlineStr">
         <is>
-          <t>$68,700.00</t>
+          <t>$66,100.00</t>
         </is>
       </c>
       <c r="AO24" s="11" t="n"/>
       <c r="AP24" s="11" t="inlineStr">
         <is>
-          <t>$30.87</t>
+          <t>$29.62</t>
         </is>
       </c>
       <c r="AQ24" s="11" t="inlineStr">
         <is>
-          <t>$46.30</t>
+          <t>$44.43</t>
         </is>
       </c>
       <c r="AR24" s="11" t="inlineStr">
@@ -55754,7 +55754,7 @@
       </c>
       <c r="AU24" s="11" t="inlineStr">
         <is>
-          <t>$66,800.00</t>
+          <t>$64,200.00</t>
         </is>
       </c>
       <c r="AV24" s="11" t="inlineStr">
@@ -55822,12 +55822,12 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>08/28/1993</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
@@ -55867,7 +55867,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>08/19/2014</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -55895,12 +55895,12 @@
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="inlineStr">
         <is>
-          <t>$16.78</t>
+          <t>$16.11</t>
         </is>
       </c>
       <c r="T25" s="13" t="inlineStr">
         <is>
-          <t>$25.17</t>
+          <t>$24.16</t>
         </is>
       </c>
       <c r="U25" s="11" t="inlineStr">
@@ -55936,12 +55936,12 @@
       <c r="AA25" s="11" t="n"/>
       <c r="AB25" s="11" t="inlineStr">
         <is>
-          <t>$16.30</t>
+          <t>$15.62</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>$24.45</t>
+          <t>$23.43</t>
         </is>
       </c>
       <c r="AD25" s="11" t="inlineStr">
@@ -55961,18 +55961,18 @@
       </c>
       <c r="AG25" s="11" t="inlineStr">
         <is>
-          <t>$35,300.00</t>
+          <t>$33,900.00</t>
         </is>
       </c>
       <c r="AH25" s="11" t="n"/>
       <c r="AI25" s="11" t="inlineStr">
         <is>
-          <t>$15.82</t>
+          <t>$15.19</t>
         </is>
       </c>
       <c r="AJ25" s="11" t="inlineStr">
         <is>
-          <t>$23.73</t>
+          <t>$22.79</t>
         </is>
       </c>
       <c r="AK25" s="11" t="inlineStr">
@@ -55992,18 +55992,18 @@
       </c>
       <c r="AN25" s="11" t="inlineStr">
         <is>
-          <t>$34,200.00</t>
+          <t>$32,900.00</t>
         </is>
       </c>
       <c r="AO25" s="11" t="n"/>
       <c r="AP25" s="11" t="inlineStr">
         <is>
-          <t>$15.34</t>
+          <t>$14.71</t>
         </is>
       </c>
       <c r="AQ25" s="11" t="inlineStr">
         <is>
-          <t>$23.01</t>
+          <t>$22.07</t>
         </is>
       </c>
       <c r="AR25" s="11" t="inlineStr">
@@ -56023,7 +56023,7 @@
       </c>
       <c r="AU25" s="11" t="inlineStr">
         <is>
-          <t>$33,200.00</t>
+          <t>$31,900.00</t>
         </is>
       </c>
       <c r="AV25" s="11" t="inlineStr">
@@ -56091,12 +56091,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>10/10/1963</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
@@ -56136,7 +56136,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>02/04/2023</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56164,12 +56164,12 @@
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="inlineStr">
         <is>
-          <t>$18.70</t>
+          <t>$17.93</t>
         </is>
       </c>
       <c r="T26" s="13" t="inlineStr">
         <is>
-          <t>$28.05</t>
+          <t>$26.89</t>
         </is>
       </c>
       <c r="U26" s="11" t="inlineStr">
@@ -56205,12 +56205,12 @@
       <c r="AA26" s="11" t="n"/>
       <c r="AB26" s="11" t="inlineStr">
         <is>
-          <t>$18.17</t>
+          <t>$17.45</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>$27.26</t>
+          <t>$26.17</t>
         </is>
       </c>
       <c r="AD26" s="11" t="inlineStr">
@@ -56230,18 +56230,18 @@
       </c>
       <c r="AG26" s="11" t="inlineStr">
         <is>
-          <t>$39,300.00</t>
+          <t>$37,800.00</t>
         </is>
       </c>
       <c r="AH26" s="11" t="n"/>
       <c r="AI26" s="11" t="inlineStr">
         <is>
-          <t>$17.64</t>
+          <t>$16.92</t>
         </is>
       </c>
       <c r="AJ26" s="11" t="inlineStr">
         <is>
-          <t>$26.46</t>
+          <t>$25.38</t>
         </is>
       </c>
       <c r="AK26" s="11" t="inlineStr">
@@ -56261,18 +56261,18 @@
       </c>
       <c r="AN26" s="11" t="inlineStr">
         <is>
-          <t>$38,200.00</t>
+          <t>$36,700.00</t>
         </is>
       </c>
       <c r="AO26" s="11" t="n"/>
       <c r="AP26" s="11" t="inlineStr">
         <is>
-          <t>$17.12</t>
+          <t>$16.44</t>
         </is>
       </c>
       <c r="AQ26" s="11" t="inlineStr">
         <is>
-          <t>$25.68</t>
+          <t>$24.66</t>
         </is>
       </c>
       <c r="AR26" s="11" t="inlineStr">
@@ -56292,7 +56292,7 @@
       </c>
       <c r="AU26" s="11" t="inlineStr">
         <is>
-          <t>$37,000.00</t>
+          <t>$35,600.00</t>
         </is>
       </c>
       <c r="AV26" s="11" t="inlineStr">
@@ -56360,7 +56360,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>07/27/1980</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
@@ -56405,7 +56405,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>08/19/2021</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56438,7 +56438,7 @@
       </c>
       <c r="T27" s="13" t="inlineStr">
         <is>
-          <t>$27.62</t>
+          <t>$26.54</t>
         </is>
       </c>
       <c r="U27" s="11" t="inlineStr">
@@ -56474,12 +56474,12 @@
       <c r="AA27" s="11" t="n"/>
       <c r="AB27" s="11" t="inlineStr">
         <is>
-          <t>$17.88</t>
+          <t>$17.16</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>$26.82</t>
+          <t>$25.74</t>
         </is>
       </c>
       <c r="AD27" s="11" t="inlineStr">
@@ -56499,18 +56499,18 @@
       </c>
       <c r="AG27" s="11" t="inlineStr">
         <is>
-          <t>$38,700.00</t>
+          <t>$37,200.00</t>
         </is>
       </c>
       <c r="AH27" s="11" t="n"/>
       <c r="AI27" s="11" t="inlineStr">
         <is>
-          <t>$17.36</t>
+          <t>$16.68</t>
         </is>
       </c>
       <c r="AJ27" s="11" t="inlineStr">
         <is>
-          <t>$26.04</t>
+          <t>$25.02</t>
         </is>
       </c>
       <c r="AK27" s="11" t="inlineStr">
@@ -56530,18 +56530,18 @@
       </c>
       <c r="AN27" s="11" t="inlineStr">
         <is>
-          <t>$37,500.00</t>
+          <t>$36,100.00</t>
         </is>
       </c>
       <c r="AO27" s="11" t="n"/>
       <c r="AP27" s="11" t="inlineStr">
         <is>
-          <t>$16.83</t>
+          <t>$16.15</t>
         </is>
       </c>
       <c r="AQ27" s="11" t="inlineStr">
         <is>
-          <t>$25.24</t>
+          <t>$24.22</t>
         </is>
       </c>
       <c r="AR27" s="11" t="inlineStr">
@@ -56561,7 +56561,7 @@
       </c>
       <c r="AU27" s="11" t="inlineStr">
         <is>
-          <t>$36,400.00</t>
+          <t>$35,000.00</t>
         </is>
       </c>
       <c r="AV27" s="11" t="inlineStr">
@@ -56629,7 +56629,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>05/09/1986</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
@@ -56674,7 +56674,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>10/22/2022</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56702,12 +56702,12 @@
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="inlineStr">
         <is>
-          <t>$14.66</t>
+          <t>$14.09</t>
         </is>
       </c>
       <c r="T28" s="13" t="inlineStr">
         <is>
-          <t>$21.99</t>
+          <t>$21.13</t>
         </is>
       </c>
       <c r="U28" s="11" t="inlineStr">
@@ -56743,12 +56743,12 @@
       <c r="AA28" s="11" t="n"/>
       <c r="AB28" s="11" t="inlineStr">
         <is>
-          <t>$14.23</t>
+          <t>$13.65</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>$21.34</t>
+          <t>$20.48</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
@@ -56768,18 +56768,18 @@
       </c>
       <c r="AG28" s="11" t="inlineStr">
         <is>
-          <t>$30,800.00</t>
+          <t>$29,600.00</t>
         </is>
       </c>
       <c r="AH28" s="11" t="n"/>
       <c r="AI28" s="11" t="inlineStr">
         <is>
-          <t>$13.80</t>
+          <t>$13.27</t>
         </is>
       </c>
       <c r="AJ28" s="11" t="inlineStr">
         <is>
-          <t>$20.70</t>
+          <t>$19.91</t>
         </is>
       </c>
       <c r="AK28" s="11" t="inlineStr">
@@ -56799,18 +56799,18 @@
       </c>
       <c r="AN28" s="11" t="inlineStr">
         <is>
-          <t>$29,800.00</t>
+          <t>$28,700.00</t>
         </is>
       </c>
       <c r="AO28" s="11" t="n"/>
       <c r="AP28" s="11" t="inlineStr">
         <is>
-          <t>$13.41</t>
+          <t>$12.88</t>
         </is>
       </c>
       <c r="AQ28" s="11" t="inlineStr">
         <is>
-          <t>$20.12</t>
+          <t>$19.32</t>
         </is>
       </c>
       <c r="AR28" s="11" t="inlineStr">
@@ -56830,7 +56830,7 @@
       </c>
       <c r="AU28" s="11" t="inlineStr">
         <is>
-          <t>$29,000.00</t>
+          <t>$27,900.00</t>
         </is>
       </c>
       <c r="AV28" s="11" t="inlineStr">
@@ -56898,12 +56898,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>12/20/1985</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56943,7 +56943,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>07/16/2016</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -56971,12 +56971,12 @@
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="inlineStr">
         <is>
-          <t>$11.92</t>
+          <t>$11.44</t>
         </is>
       </c>
       <c r="T29" s="13" t="inlineStr">
         <is>
-          <t>$17.88</t>
+          <t>$17.16</t>
         </is>
       </c>
       <c r="U29" s="11" t="inlineStr">
@@ -57012,12 +57012,12 @@
       <c r="AA29" s="11" t="n"/>
       <c r="AB29" s="11" t="inlineStr">
         <is>
-          <t>$11.59</t>
+          <t>$11.11</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>$17.38</t>
+          <t>$16.66</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
@@ -57037,18 +57037,18 @@
       </c>
       <c r="AG29" s="11" t="inlineStr">
         <is>
-          <t>$25,100.00</t>
+          <t>$24,100.00</t>
         </is>
       </c>
       <c r="AH29" s="11" t="n"/>
       <c r="AI29" s="11" t="inlineStr">
         <is>
-          <t>$11.25</t>
+          <t>$10.82</t>
         </is>
       </c>
       <c r="AJ29" s="11" t="inlineStr">
         <is>
-          <t>$16.88</t>
+          <t>$16.23</t>
         </is>
       </c>
       <c r="AK29" s="11" t="inlineStr">
@@ -57068,18 +57068,18 @@
       </c>
       <c r="AN29" s="11" t="inlineStr">
         <is>
-          <t>$24,300.00</t>
+          <t>$23,400.00</t>
         </is>
       </c>
       <c r="AO29" s="11" t="n"/>
       <c r="AP29" s="11" t="inlineStr">
         <is>
-          <t>$10.91</t>
+          <t>$10.48</t>
         </is>
       </c>
       <c r="AQ29" s="11" t="inlineStr">
         <is>
-          <t>$16.37</t>
+          <t>$15.72</t>
         </is>
       </c>
       <c r="AR29" s="11" t="inlineStr">
@@ -57099,7 +57099,7 @@
       </c>
       <c r="AU29" s="11" t="inlineStr">
         <is>
-          <t>$23,600.00</t>
+          <t>$22,700.00</t>
         </is>
       </c>
       <c r="AV29" s="11" t="inlineStr">
@@ -57167,12 +57167,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>06/14/1991</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57212,7 +57212,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>06/14/2018</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57240,12 +57240,12 @@
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="inlineStr">
         <is>
-          <t>$28.85</t>
+          <t>$27.69</t>
         </is>
       </c>
       <c r="T30" s="13" t="inlineStr">
         <is>
-          <t>$43.28</t>
+          <t>$41.54</t>
         </is>
       </c>
       <c r="U30" s="11" t="inlineStr">
@@ -57281,12 +57281,12 @@
       <c r="AA30" s="11" t="n"/>
       <c r="AB30" s="11" t="inlineStr">
         <is>
-          <t>$28.03</t>
+          <t>$26.92</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>$42.05</t>
+          <t>$40.38</t>
         </is>
       </c>
       <c r="AD30" s="11" t="inlineStr">
@@ -57306,18 +57306,18 @@
       </c>
       <c r="AG30" s="11" t="inlineStr">
         <is>
-          <t>$60,600.00</t>
+          <t>$58,300.00</t>
         </is>
       </c>
       <c r="AH30" s="11" t="n"/>
       <c r="AI30" s="11" t="inlineStr">
         <is>
-          <t>$27.21</t>
+          <t>$26.11</t>
         </is>
       </c>
       <c r="AJ30" s="11" t="inlineStr">
         <is>
-          <t>$40.81</t>
+          <t>$39.16</t>
         </is>
       </c>
       <c r="AK30" s="11" t="inlineStr">
@@ -57337,18 +57337,18 @@
       </c>
       <c r="AN30" s="11" t="inlineStr">
         <is>
-          <t>$58,900.00</t>
+          <t>$56,600.00</t>
         </is>
       </c>
       <c r="AO30" s="11" t="n"/>
       <c r="AP30" s="11" t="inlineStr">
         <is>
-          <t>$26.44</t>
+          <t>$25.38</t>
         </is>
       </c>
       <c r="AQ30" s="11" t="inlineStr">
         <is>
-          <t>$39.66</t>
+          <t>$38.07</t>
         </is>
       </c>
       <c r="AR30" s="11" t="inlineStr">
@@ -57368,7 +57368,7 @@
       </c>
       <c r="AU30" s="11" t="inlineStr">
         <is>
-          <t>$57,200.00</t>
+          <t>$55,000.00</t>
         </is>
       </c>
       <c r="AV30" s="11" t="inlineStr">
@@ -57436,7 +57436,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>09/13/1994</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -57481,7 +57481,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>10/23/2014</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57509,12 +57509,12 @@
       <c r="R31" s="14" t="n"/>
       <c r="S31" s="14" t="inlineStr">
         <is>
-          <t>$27.93</t>
+          <t>$26.83</t>
         </is>
       </c>
       <c r="T31" s="13" t="inlineStr">
         <is>
-          <t>$41.89</t>
+          <t>$40.24</t>
         </is>
       </c>
       <c r="U31" s="11" t="inlineStr">
@@ -57550,12 +57550,12 @@
       <c r="AA31" s="11" t="n"/>
       <c r="AB31" s="11" t="inlineStr">
         <is>
-          <t>$27.12</t>
+          <t>$26.01</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>$40.68</t>
+          <t>$39.02</t>
         </is>
       </c>
       <c r="AD31" s="11" t="inlineStr">
@@ -57575,18 +57575,18 @@
       </c>
       <c r="AG31" s="11" t="inlineStr">
         <is>
-          <t>$58,700.00</t>
+          <t>$56,400.00</t>
         </is>
       </c>
       <c r="AH31" s="11" t="n"/>
       <c r="AI31" s="11" t="inlineStr">
         <is>
-          <t>$26.35</t>
+          <t>$25.29</t>
         </is>
       </c>
       <c r="AJ31" s="11" t="inlineStr">
         <is>
-          <t>$39.53</t>
+          <t>$37.94</t>
         </is>
       </c>
       <c r="AK31" s="11" t="inlineStr">
@@ -57606,18 +57606,18 @@
       </c>
       <c r="AN31" s="11" t="inlineStr">
         <is>
-          <t>$57,000.00</t>
+          <t>$54,800.00</t>
         </is>
       </c>
       <c r="AO31" s="11" t="n"/>
       <c r="AP31" s="11" t="inlineStr">
         <is>
-          <t>$25.58</t>
+          <t>$24.57</t>
         </is>
       </c>
       <c r="AQ31" s="11" t="inlineStr">
         <is>
-          <t>$38.37</t>
+          <t>$36.86</t>
         </is>
       </c>
       <c r="AR31" s="11" t="inlineStr">
@@ -57637,7 +57637,7 @@
       </c>
       <c r="AU31" s="11" t="inlineStr">
         <is>
-          <t>$55,300.00</t>
+          <t>$53,200.00</t>
         </is>
       </c>
       <c r="AV31" s="11" t="inlineStr">
@@ -57705,7 +57705,7 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>03/23/1976</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
@@ -57750,7 +57750,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>08/17/2017</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57778,12 +57778,12 @@
       <c r="R32" s="14" t="n"/>
       <c r="S32" s="14" t="inlineStr">
         <is>
-          <t>$13.22</t>
+          <t>$12.69</t>
         </is>
       </c>
       <c r="T32" s="13" t="inlineStr">
         <is>
-          <t>$19.83</t>
+          <t>$19.04</t>
         </is>
       </c>
       <c r="U32" s="11" t="inlineStr">
@@ -57819,12 +57819,12 @@
       <c r="AA32" s="11" t="n"/>
       <c r="AB32" s="11" t="inlineStr">
         <is>
-          <t>$12.84</t>
+          <t>$12.31</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>$19.26</t>
+          <t>$18.46</t>
         </is>
       </c>
       <c r="AD32" s="11" t="inlineStr">
@@ -57844,18 +57844,18 @@
       </c>
       <c r="AG32" s="11" t="inlineStr">
         <is>
-          <t>$27,800.00</t>
+          <t>$26,700.00</t>
         </is>
       </c>
       <c r="AH32" s="11" t="n"/>
       <c r="AI32" s="11" t="inlineStr">
         <is>
-          <t>$12.45</t>
+          <t>$11.97</t>
         </is>
       </c>
       <c r="AJ32" s="11" t="inlineStr">
         <is>
-          <t>$18.67</t>
+          <t>$17.96</t>
         </is>
       </c>
       <c r="AK32" s="11" t="inlineStr">
@@ -57875,18 +57875,18 @@
       </c>
       <c r="AN32" s="11" t="inlineStr">
         <is>
-          <t>$26,900.00</t>
+          <t>$25,900.00</t>
         </is>
       </c>
       <c r="AO32" s="11" t="n"/>
       <c r="AP32" s="11" t="inlineStr">
         <is>
-          <t>$12.07</t>
+          <t>$11.59</t>
         </is>
       </c>
       <c r="AQ32" s="11" t="inlineStr">
         <is>
-          <t>$18.11</t>
+          <t>$17.38</t>
         </is>
       </c>
       <c r="AR32" s="11" t="inlineStr">
@@ -57906,7 +57906,7 @@
       </c>
       <c r="AU32" s="11" t="inlineStr">
         <is>
-          <t>$26,100.00</t>
+          <t>$25,100.00</t>
         </is>
       </c>
       <c r="AV32" s="11" t="inlineStr">
@@ -57974,7 +57974,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>01/01/1986</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
@@ -58019,7 +58019,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>01/01/2019</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58047,12 +58047,12 @@
       <c r="R33" s="14" t="n"/>
       <c r="S33" s="14" t="inlineStr">
         <is>
-          <t>$10.82</t>
+          <t>$10.38</t>
         </is>
       </c>
       <c r="T33" s="13" t="inlineStr">
         <is>
-          <t>$16.23</t>
+          <t>$15.57</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -58088,12 +58088,12 @@
       <c r="AA33" s="11" t="n"/>
       <c r="AB33" s="11" t="inlineStr">
         <is>
-          <t>$10.48</t>
+          <t>$10.05</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>$15.72</t>
+          <t>$15.08</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
@@ -58113,18 +58113,18 @@
       </c>
       <c r="AG33" s="11" t="inlineStr">
         <is>
-          <t>$22,700.00</t>
+          <t>$21,800.00</t>
         </is>
       </c>
       <c r="AH33" s="11" t="n"/>
       <c r="AI33" s="11" t="inlineStr">
         <is>
-          <t>$10.19</t>
+          <t>$9.81</t>
         </is>
       </c>
       <c r="AJ33" s="11" t="inlineStr">
         <is>
-          <t>$15.29</t>
+          <t>$14.71</t>
         </is>
       </c>
       <c r="AK33" s="11" t="inlineStr">
@@ -58144,18 +58144,18 @@
       </c>
       <c r="AN33" s="11" t="inlineStr">
         <is>
-          <t>$22,000.00</t>
+          <t>$21,200.00</t>
         </is>
       </c>
       <c r="AO33" s="11" t="n"/>
       <c r="AP33" s="11" t="inlineStr">
         <is>
-          <t>$9.90</t>
+          <t>$9.52</t>
         </is>
       </c>
       <c r="AQ33" s="11" t="inlineStr">
         <is>
-          <t>$14.85</t>
+          <t>$14.28</t>
         </is>
       </c>
       <c r="AR33" s="11" t="inlineStr">
@@ -58175,7 +58175,7 @@
       </c>
       <c r="AU33" s="11" t="inlineStr">
         <is>
-          <t>$21,400.00</t>
+          <t>$20,600.00</t>
         </is>
       </c>
       <c r="AV33" s="11" t="inlineStr">
@@ -58243,7 +58243,7 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>01/25/1994</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
@@ -58288,7 +58288,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>04/09/2024</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58316,12 +58316,12 @@
       <c r="R34" s="14" t="n"/>
       <c r="S34" s="14" t="inlineStr">
         <is>
-          <t>$14.62</t>
+          <t>$14.04</t>
         </is>
       </c>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>$21.93</t>
+          <t>$21.06</t>
         </is>
       </c>
       <c r="U34" s="11" t="inlineStr">
@@ -58357,12 +58357,12 @@
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="11" t="inlineStr">
         <is>
-          <t>$14.18</t>
+          <t>$13.61</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>$21.27</t>
+          <t>$20.41</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
@@ -58382,18 +58382,18 @@
       </c>
       <c r="AG34" s="11" t="inlineStr">
         <is>
-          <t>$30,700.00</t>
+          <t>$29,500.00</t>
         </is>
       </c>
       <c r="AH34" s="11" t="n"/>
       <c r="AI34" s="11" t="inlineStr">
         <is>
-          <t>$13.75</t>
+          <t>$13.22</t>
         </is>
       </c>
       <c r="AJ34" s="11" t="inlineStr">
         <is>
-          <t>$20.62</t>
+          <t>$19.83</t>
         </is>
       </c>
       <c r="AK34" s="11" t="inlineStr">
@@ -58413,18 +58413,18 @@
       </c>
       <c r="AN34" s="11" t="inlineStr">
         <is>
-          <t>$29,700.00</t>
+          <t>$28,600.00</t>
         </is>
       </c>
       <c r="AO34" s="11" t="n"/>
       <c r="AP34" s="11" t="inlineStr">
         <is>
-          <t>$13.37</t>
+          <t>$12.84</t>
         </is>
       </c>
       <c r="AQ34" s="11" t="inlineStr">
         <is>
-          <t>$20.05</t>
+          <t>$19.26</t>
         </is>
       </c>
       <c r="AR34" s="11" t="inlineStr">
@@ -58444,7 +58444,7 @@
       </c>
       <c r="AU34" s="11" t="inlineStr">
         <is>
-          <t>$28,900.00</t>
+          <t>$27,800.00</t>
         </is>
       </c>
       <c r="AV34" s="11" t="inlineStr">
@@ -58512,7 +58512,7 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>05/10/1990</t>
+          <t>03/03/2000</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
@@ -58557,7 +58557,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>03/02/2020</t>
+          <t>01/01/2015</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -58585,12 +58585,12 @@
       <c r="R35" s="14" t="n"/>
       <c r="S35" s="14" t="inlineStr">
         <is>
-          <t>$65.67</t>
+          <t>$63.03</t>
         </is>
       </c>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>$98.50</t>
+          <t>$94.55</t>
         </is>
       </c>
       <c r="U35" s="11" t="inlineStr">
@@ -58626,12 +58626,12 @@
       <c r="AA35" s="11" t="n"/>
       <c r="AB35" s="11" t="inlineStr">
         <is>
-          <t>$63.75</t>
+          <t>$61.20</t>
         </is>
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>$95.62</t>
+          <t>$91.80</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
@@ -58651,18 +58651,18 @@
       </c>
       <c r="AG35" s="11" t="inlineStr">
         <is>
-          <t>$137,900.00</t>
+          <t>$132,600.00</t>
         </is>
       </c>
       <c r="AH35" s="11" t="n"/>
       <c r="AI35" s="11" t="inlineStr">
         <is>
-          <t>$61.88</t>
+          <t>$59.42</t>
         </is>
       </c>
       <c r="AJ35" s="11" t="inlineStr">
         <is>
-          <t>$92.82</t>
+          <t>$89.13</t>
         </is>
       </c>
       <c r="AK35" s="11" t="inlineStr">
@@ -58682,18 +58682,18 @@
       </c>
       <c r="AN35" s="11" t="inlineStr">
         <is>
-          <t>$133,800.00</t>
+          <t>$128,700.00</t>
         </is>
       </c>
       <c r="AO35" s="11" t="n"/>
       <c r="AP35" s="11" t="inlineStr">
         <is>
-          <t>$60.10</t>
+          <t>$57.69</t>
         </is>
       </c>
       <c r="AQ35" s="11" t="inlineStr">
         <is>
-          <t>$90.15</t>
+          <t>$86.53</t>
         </is>
       </c>
       <c r="AR35" s="11" t="inlineStr">
@@ -58713,7 +58713,7 @@
       </c>
       <c r="AU35" s="11" t="inlineStr">
         <is>
-          <t>$130,000.00</t>
+          <t>$125,000.00</t>
         </is>
       </c>
       <c r="AV35" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat(data): provenance in the downloads and on the sample table
The .xlsx and .csv downloads carried no lineage — someone with the file could
not tell which sources or vintages produced it. The on-page sample table had the
same gap: 59 census columns, no indication of where each value came from.

- every workbook now ships a PROVENANCE sheet listing each source, its warehouse
  table, row count, vintage and what it feeds, read LIVE from the warehouse at
  generation time. It is a second sheet, so the census sheet stays a faithful
  client shape (the real 59 ND3 columns, nothing added).
- sample-rows table labels each reference-drawn column beneath its header
  (O*NET for title/SOC, BLS OEWS for wage figures, Census/ZCTA for state + ZIP)
- refreshed the downloadable fixtures to the current generation
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -8,9 +8,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority Census Template" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Census Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROVENANCE" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
@@ -33,6 +33,7 @@
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId24"/>
     <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId25"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId26"/>
   </externalReferences>
   <definedNames>
     <definedName name="_____dc1" hidden="1">{#N/A,#N/A,FALSE,"COVER PAGE";#N/A,#N/A,FALSE,"HIGHLITES";#N/A,#N/A,FALSE,"INC STATE (1)";#N/A,#N/A,FALSE,"DPC BY DEPT";#N/A,#N/A,FALSE,"FIXED COSTS";#N/A,#N/A,FALSE,"PRODUCTION";#N/A,#N/A,FALSE,"SALES TRND";#N/A,#N/A,FALSE,"BALANCE SHEET";#N/A,#N/A,FALSE,"INVENTORY";#N/A,#N/A,FALSE,"MFG VAR";#N/A,#N/A,FALSE,"OVRHD SPND";#N/A,#N/A,FALSE,"ENERGY COSTS";#N/A,#N/A,FALSE,"MAINTENANCE";#N/A,#N/A,FALSE,"LABOR";#N/A,#N/A,FALSE,"ACTVSFORECAST"}</definedName>
@@ -53931,12 +53932,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>10/22/1991</t>
+          <t>05/13/1970</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53976,7 +53977,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>04/08/2022</t>
+          <t>06/14/2023</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54200,12 +54201,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>09/05/1962</t>
+          <t>12/04/1997</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -54245,7 +54246,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>05/11/2023</t>
+          <t>09/20/2014</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54469,7 +54470,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>05/05/1982</t>
+          <t>03/07/1992</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -54514,7 +54515,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>01/02/2020</t>
+          <t>09/21/2014</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54799,7 +54800,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>05/11/2019</t>
+          <t>05/11/2023</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55023,12 +55024,12 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>09/13/1986</t>
+          <t>08/24/1973</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
@@ -55068,7 +55069,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>10/23/2013</t>
+          <t>12/27/2017</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55557,7 +55558,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>09/05/1994</t>
+          <t>09/09/1966</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -55598,7 +55599,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>05/11/2018</t>
+          <t>02/03/2021</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55822,7 +55823,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>08/28/1993</t>
+          <t>02/02/1963</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
@@ -55867,7 +55868,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>08/19/2014</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -56091,12 +56092,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>10/10/1963</t>
+          <t>01/13/1966</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
@@ -56136,7 +56137,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>02/04/2023</t>
+          <t>02/05/2021</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56360,7 +56361,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>07/27/1980</t>
+          <t>07/23/1964</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
@@ -56405,7 +56406,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>08/19/2021</t>
+          <t>12/27/2024</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56629,12 +56630,12 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>05/09/1986</t>
+          <t>08/28/2001</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
@@ -56674,7 +56675,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>10/22/2022</t>
+          <t>08/19/2022</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56898,12 +56899,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>12/20/1985</t>
+          <t>09/13/1998</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56943,7 +56944,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>07/16/2016</t>
+          <t>10/23/2018</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -57167,12 +57168,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>06/14/1991</t>
+          <t>03/07/1984</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57212,7 +57213,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>06/14/2018</t>
+          <t>09/21/2024</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57436,7 +57437,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>09/13/1994</t>
+          <t>03/27/1964</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -57481,7 +57482,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>10/23/2014</t>
+          <t>04/09/2016</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57705,12 +57706,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>03/23/1976</t>
+          <t>12/28/1997</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -57750,7 +57751,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>08/17/2017</t>
+          <t>12/28/2024</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57974,7 +57975,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>01/01/1986</t>
+          <t>09/25/1966</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
@@ -58019,7 +58020,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>01/01/2019</t>
+          <t>12/27/2016</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58243,12 +58244,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>01/25/1994</t>
+          <t>06/22/1967</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
@@ -58288,7 +58289,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>04/09/2024</t>
+          <t>12/26/2014</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58512,12 +58513,12 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>03/03/2000</t>
+          <t>02/02/1987</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
@@ -58557,7 +58558,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>01/01/2015</t>
+          <t>01/01/2022</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -65425,4 +65426,471 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Nine Dean — simulated census: data provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>generated 2026-07-20 00:02 from the reference warehouse (public.ext_*)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>warehouse table</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>vintage</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>feeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MIT · Living Wage Calculator</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ext_mit_expense</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>301,824</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>mit:livingwage.mit.edu:2026</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Engine A basket components</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MIT · Living Wage Calculator</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ext_mit_living_wage</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>113,184</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>mit:livingwage.mit.edu:2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Engine A living-wage reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EPI · Family Budget Calculator</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ext_epi_cost</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>502,880</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>epi:2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Engine A basket (food, childcare, medical, housing, other)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EPI · Family Budget Calculator</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ext_epi_county</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3,143</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>epi:2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Engine A county coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ACS · B25064 median gross rent</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ext_acs</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3,222</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>acs:5y2023-B25064</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Engine A housing candidate</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CNT · H+T Affordability Index</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ext_cnt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>3,144</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>cnt:2022</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Engine A transportation (override, not MAX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BLS OEWS · state wages</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ext_bls_oews_state_wage</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>35,427</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>May2024</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>wages by state+SOC (p10/p25/median); prevailing-wage overlay</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>O*NET · SOC occupations</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ext_onet_soc_occupation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1,016</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>O*NET 29.0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>job titles and SOC codes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>O*NET · SOC alternate titles</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ext_onet_soc_alt_title</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>55,119</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>O*NET 29.0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>title → SOC matching</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Census · ZCTA↔county crosswalk</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ext_census_zcta_county</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>23,355</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>census_zcta:2020</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>residence ZIP → county</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Census · county gazetteer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ext_census_county</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>3,222</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>census_county:2024</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>county names / states</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A Better Balance · PSL statutes</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ext_abb_psl_law</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>abb:2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Engine B floors (cap / preempted / no-cap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KFF · EHBS benchmarks</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ext_kff_ehbs_health_benchmarks</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>kff_ehbs:2025</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Engine C employer-contribution thresholds</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Peterson-KFF · OOP cost-sharing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ext_peterson_kff_oop_costsharing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>live scrape; page modified 2026-02-11</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Engine C out-of-pocket exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PolicyEngine US</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>in-process library (not a warehouse table)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>policyengine-us 1.745.0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Engine A federal + state + payroll + local tax</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(data): implausible birth and hire dates in the census
Reviewing the sample rows surfaced two defects in the generated demographics:

- 11 of 300 employees were hired UNDER 16 (youngest 13.3). DOB and hire date
  were derived independently from one seed with no constraint between them.
- 12 rows had a hire date whose month/day mirrored the birthday, because both
  used the same seed arithmetic.

Hire year is now floored at birth_year+19 (the +19 absorbs a birthday falling
after the hire date) and the hire month/day is offset off a different part of
the seed.

Verified across all 300 rows: 0 hired under 18, 0 future hire dates,
0 mirrored month/days, ages 19-61 with a median of 37.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53932,12 +53932,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>05/13/1970</t>
+          <t>02/22/1963</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53977,7 +53977,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>06/14/2023</t>
+          <t>10/16/2017</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54201,7 +54201,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>12/04/1997</t>
+          <t>04/04/1993</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -54246,7 +54246,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>09/20/2014</t>
+          <t>11/24/2025</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54470,7 +54470,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>03/07/1992</t>
+          <t>01/13/1966</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -54515,7 +54515,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>09/21/2014</t>
+          <t>06/03/2020</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54755,12 +54755,12 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>09/05/1970</t>
+          <t>02/14/1967</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -54800,7 +54800,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>05/11/2023</t>
+          <t>07/07/2024</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55024,12 +55024,12 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>08/24/1973</t>
+          <t>03/03/1972</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
@@ -55069,7 +55069,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>12/27/2017</t>
+          <t>10/13/2012</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55334,7 +55334,7 @@
       </c>
       <c r="K23" s="14" t="inlineStr">
         <is>
-          <t>01/01/2012</t>
+          <t>05/07/2012</t>
         </is>
       </c>
       <c r="L23" s="14" t="n"/>
@@ -55558,7 +55558,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>09/09/1966</t>
+          <t>11/07/1972</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -55599,7 +55599,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>02/03/2021</t>
+          <t>07/20/2017</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55823,12 +55823,12 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>02/02/1963</t>
+          <t>01/21/1986</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
@@ -55868,7 +55868,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>11/04/2013</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -56092,12 +56092,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>01/13/1966</t>
+          <t>02/14/1979</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
@@ -56137,7 +56137,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>02/05/2021</t>
+          <t>07/06/2019</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56361,12 +56361,12 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>07/23/1964</t>
+          <t>12/20/1997</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
@@ -56406,7 +56406,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>12/27/2024</t>
+          <t>07/13/2020</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56630,12 +56630,12 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>08/28/2001</t>
+          <t>07/19/1976</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
@@ -56675,7 +56675,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>08/19/2022</t>
+          <t>01/28/2012</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56899,12 +56899,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>09/13/1998</t>
+          <t>06/26/1971</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56944,7 +56944,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>10/23/2018</t>
+          <t>05/08/2020</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -57168,12 +57168,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>03/07/1984</t>
+          <t>06/10/1975</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57213,7 +57213,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>09/21/2024</t>
+          <t>04/20/2021</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57437,12 +57437,12 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>03/27/1964</t>
+          <t>10/06/1995</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -57482,7 +57482,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>04/09/2016</t>
+          <t>03/26/2017</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57706,12 +57706,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>12/28/1997</t>
+          <t>07/27/1972</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -57751,7 +57751,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>12/28/2024</t>
+          <t>03/19/2014</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57975,7 +57975,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>09/25/1966</t>
+          <t>05/05/1970</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
@@ -58020,7 +58020,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>12/27/2016</t>
+          <t>09/19/2014</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58244,12 +58244,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>06/22/1967</t>
+          <t>03/27/1980</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
@@ -58289,7 +58289,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>12/26/2014</t>
+          <t>07/20/2020</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58513,12 +58513,12 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>02/02/1987</t>
+          <t>07/27/1972</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
@@ -58558,7 +58558,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>01/01/2022</t>
+          <t>03/16/2024</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -65454,7 +65454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-20 00:02 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-20 00:26 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(data): expectations CSV now identifies the employee
The .csv download carried only (code, edge_id, expected_behavior), so a reader
had to open the workbook to see WHICH employee an expectation referred to — and
the E3 case, which deliberately blanks the Code, had nothing identifying it at
all beyond '(blank)'.

Added soc_code, title, work_state, residence_zip, employment_classification,
exempt and total_comp_2026 — enough to read the CSV on its own without
duplicating all 59 columns.

E3 now reads '(blank) | 13-1051 Warehouse Lead | TX | $40,000'. E4 stays empty
by design: it is the fully-empty padding row.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53932,12 +53932,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>02/22/1963</t>
+          <t>07/03/1968</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53977,7 +53977,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>10/16/2017</t>
+          <t>12/10/2014</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54201,12 +54201,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>04/04/1993</t>
+          <t>11/11/1980</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -54246,7 +54246,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>11/24/2025</t>
+          <t>10/04/2019</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54470,12 +54470,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>01/13/1966</t>
+          <t>12/20/2001</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -54515,7 +54515,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>06/03/2020</t>
+          <t>04/26/2022</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54755,7 +54755,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>02/14/1967</t>
+          <t>06/10/1963</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
@@ -54800,7 +54800,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>07/07/2024</t>
+          <t>04/25/2014</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55024,12 +55024,12 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>03/03/1972</t>
+          <t>04/16/1965</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
@@ -55069,7 +55069,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>10/13/2012</t>
+          <t>10/22/2024</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55558,12 +55558,12 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>11/07/1972</t>
+          <t>06/10/1999</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -55599,7 +55599,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>07/20/2017</t>
+          <t>01/03/2018</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55823,7 +55823,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>01/21/1986</t>
+          <t>03/07/1972</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
@@ -55868,7 +55868,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>11/04/2013</t>
+          <t>12/16/2021</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -56092,12 +56092,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>02/14/1979</t>
+          <t>11/07/1976</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
@@ -56137,7 +56137,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>07/06/2019</t>
+          <t>04/15/2012</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56361,12 +56361,12 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>12/20/1997</t>
+          <t>01/21/1966</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
@@ -56406,7 +56406,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>07/13/2020</t>
+          <t>08/11/2013</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56630,7 +56630,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>07/19/1976</t>
+          <t>07/11/1964</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
@@ -56675,7 +56675,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>01/28/2012</t>
+          <t>02/19/2021</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56899,12 +56899,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>06/26/1971</t>
+          <t>05/25/1970</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56944,7 +56944,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>05/08/2020</t>
+          <t>04/07/2020</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -57168,12 +57168,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>06/10/1975</t>
+          <t>05/01/1962</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57213,7 +57213,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>04/20/2021</t>
+          <t>01/12/2019</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57437,7 +57437,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>10/06/1995</t>
+          <t>04/24/1977</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -57482,7 +57482,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>03/26/2017</t>
+          <t>12/04/2016</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57706,12 +57706,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>07/27/1972</t>
+          <t>08/12/1993</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -57751,7 +57751,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>03/19/2014</t>
+          <t>03/03/2021</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57975,7 +57975,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>05/05/1970</t>
+          <t>03/19/1976</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
@@ -58020,7 +58020,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>09/19/2014</t>
+          <t>08/03/2022</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58289,7 +58289,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>07/20/2020</t>
+          <t>01/12/2014</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58513,7 +58513,7 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>07/27/1972</t>
+          <t>07/03/1996</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
@@ -58558,7 +58558,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>03/16/2024</t>
+          <t>03/16/2018</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -65454,7 +65454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-20 00:26 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-20 12:57 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(data): ship fixtures carrying a company name, and show it on each card
The workbooks served for download had an empty 'Company Name:' header
cell, so a downloaded file gave no clue which acquisition target it
represented. Re-synced from the backend generator, which now stamps a
distinct fictional target and a generation date into every file.

The card also shows the name, so the files are distinguishable before
downloading rather than only after opening one.

The name lives in the component rather than Supabase content: it is a
caption for a static asset, and three migrations are already pending
without adding a fourth for a label.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53075,7 +53075,11 @@
           <t>Company Name:</t>
         </is>
       </c>
-      <c r="B8" s="46" t="n"/>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>Composite Diligence Target (all edge cases)</t>
+        </is>
+      </c>
       <c r="C8" s="46" t="n"/>
       <c r="D8" s="46" t="n"/>
       <c r="E8" s="45" t="n"/>
@@ -53140,7 +53144,11 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B9" s="43" t="n"/>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>07/20/2026</t>
+        </is>
+      </c>
       <c r="C9" s="43" t="n"/>
       <c r="D9" s="43" t="n"/>
       <c r="E9" s="43" t="n"/>
@@ -53932,7 +53940,7 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>07/03/1968</t>
+          <t>03/15/1976</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
@@ -53977,7 +53985,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>12/10/2014</t>
+          <t>09/01/2014</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54201,7 +54209,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>11/11/1980</t>
+          <t>05/01/1994</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -54246,7 +54254,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>10/04/2019</t>
+          <t>04/07/2013</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54470,12 +54478,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>12/20/2001</t>
+          <t>05/05/1998</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -54515,7 +54523,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>04/26/2022</t>
+          <t>12/18/2018</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54755,12 +54763,12 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>06/10/1963</t>
+          <t>07/23/1980</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -54800,7 +54808,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>04/25/2014</t>
+          <t>04/03/2019</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55024,7 +55032,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>04/16/1965</t>
+          <t>08/08/1993</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -55069,7 +55077,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>10/22/2024</t>
+          <t>01/21/2021</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55558,7 +55566,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>06/10/1999</t>
+          <t>12/16/1969</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -55599,7 +55607,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>01/03/2018</t>
+          <t>11/05/2014</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55823,7 +55831,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>03/07/1972</t>
+          <t>01/17/1970</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
@@ -55868,7 +55876,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>12/16/2021</t>
+          <t>09/27/2022</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -56092,7 +56100,7 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>11/07/1976</t>
+          <t>03/23/1980</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
@@ -56137,7 +56145,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>04/15/2012</t>
+          <t>02/17/2025</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56361,12 +56369,12 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>01/21/1966</t>
+          <t>12/28/1977</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
@@ -56406,7 +56414,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>08/11/2013</t>
+          <t>06/12/2024</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56630,12 +56638,12 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>07/11/1964</t>
+          <t>02/10/1975</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
@@ -56675,7 +56683,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>02/19/2021</t>
+          <t>11/24/2017</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56899,12 +56907,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>05/25/1970</t>
+          <t>02/18/1995</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56944,7 +56952,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>04/07/2020</t>
+          <t>01/02/2017</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -57168,7 +57176,7 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>05/01/1962</t>
+          <t>11/03/1984</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
@@ -57213,7 +57221,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>01/12/2019</t>
+          <t>11/25/2024</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57437,12 +57445,12 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>04/24/1977</t>
+          <t>03/15/2000</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -57482,7 +57490,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>12/04/2016</t>
+          <t>03/22/2022</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57706,12 +57714,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>08/12/1993</t>
+          <t>03/19/1972</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -57751,7 +57759,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>03/03/2021</t>
+          <t>08/10/2016</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57975,12 +57983,12 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>03/19/1976</t>
+          <t>10/02/1991</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D33" s="21" t="inlineStr">
@@ -58020,7 +58028,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>08/03/2022</t>
+          <t>04/17/2018</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58244,7 +58252,7 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>03/27/1980</t>
+          <t>05/09/1990</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
@@ -58289,7 +58297,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>01/12/2014</t>
+          <t>03/18/2014</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58513,7 +58521,7 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>07/03/1996</t>
+          <t>07/07/1980</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
@@ -58558,7 +58566,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>03/16/2018</t>
+          <t>05/13/2020</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -65454,7 +65462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-20 12:57 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-20 18:20 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(data): ship E28 (derived SOC) and refresh the affected row counts
Adds the edge case for a census that supplies no SOC code, and
re-syncs the fixture workbooks so the downloadable edge_ingestion.xlsx
carries the new row.

E28's description states the full rule, not just the fallback: a
census-supplied code always wins and is cross-checked against the title
(soc_title_agrees); a blank derives from the title; a near-tied second
occupation is surfaced as a rival with its confidence rather than
silently chosen; no match yields soc_source=unmatched, never a stub.

edge_ingestion 7->8 rows, all_combined 17->18.

Verified the migration chain in order on a scratch Postgres 16: E28
appends to the ingestion group, existing items are preserved, counts
update.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53940,7 +53940,7 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>03/15/1976</t>
+          <t>09/21/1974</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
@@ -53985,7 +53985,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>09/01/2014</t>
+          <t>06/04/2013</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54209,12 +54209,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>05/01/1994</t>
+          <t>08/12/1989</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -54254,7 +54254,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>04/07/2013</t>
+          <t>06/01/2021</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54478,12 +54478,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>05/05/1998</t>
+          <t>04/24/1997</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -54523,7 +54523,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>12/18/2018</t>
+          <t>12/06/2018</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54763,7 +54763,7 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>07/23/1980</t>
+          <t>03/19/1972</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
@@ -54808,7 +54808,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>04/03/2019</t>
+          <t>08/13/2020</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55032,7 +55032,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>08/08/1993</t>
+          <t>02/14/1995</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -55077,7 +55077,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>01/21/2021</t>
+          <t>07/23/2025</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55566,7 +55566,7 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>12/16/1969</t>
+          <t>08/04/1981</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
@@ -55587,7 +55587,7 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>15-2021</t>
+          <t>39-4031</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
@@ -55597,7 +55597,7 @@
       </c>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>Mathematicians</t>
+          <t>Morticians, Undertakers, and Funeral Arrangers</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
@@ -55607,7 +55607,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>11/05/2014</t>
+          <t>07/12/2012</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55635,12 +55635,12 @@
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="inlineStr">
         <is>
-          <t>$32.36</t>
+          <t>$13.03</t>
         </is>
       </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
-          <t>$48.54</t>
+          <t>$19.54</t>
         </is>
       </c>
       <c r="U24" s="11" t="inlineStr">
@@ -55660,7 +55660,7 @@
       </c>
       <c r="X24" s="11" t="inlineStr">
         <is>
-          <t>$2,800.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="Y24" s="11" t="inlineStr">
@@ -55670,18 +55670,18 @@
       </c>
       <c r="Z24" s="11" t="inlineStr">
         <is>
-          <t>$70,100.00</t>
+          <t>$28,200.00</t>
         </is>
       </c>
       <c r="AA24" s="11" t="n"/>
       <c r="AB24" s="11" t="inlineStr">
         <is>
-          <t>$31.44</t>
+          <t>$12.64</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>$47.16</t>
+          <t>$18.96</t>
         </is>
       </c>
       <c r="AD24" s="11" t="inlineStr">
@@ -55691,7 +55691,7 @@
       </c>
       <c r="AE24" s="11" t="inlineStr">
         <is>
-          <t>$2,700.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AF24" s="11" t="inlineStr">
@@ -55701,18 +55701,18 @@
       </c>
       <c r="AG24" s="11" t="inlineStr">
         <is>
-          <t>$68,100.00</t>
+          <t>$27,400.00</t>
         </is>
       </c>
       <c r="AH24" s="11" t="n"/>
       <c r="AI24" s="11" t="inlineStr">
         <is>
-          <t>$30.53</t>
+          <t>$12.26</t>
         </is>
       </c>
       <c r="AJ24" s="11" t="inlineStr">
         <is>
-          <t>$45.80</t>
+          <t>$18.39</t>
         </is>
       </c>
       <c r="AK24" s="11" t="inlineStr">
@@ -55722,7 +55722,7 @@
       </c>
       <c r="AL24" s="11" t="inlineStr">
         <is>
-          <t>$2,600.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AM24" s="11" t="inlineStr">
@@ -55732,18 +55732,18 @@
       </c>
       <c r="AN24" s="11" t="inlineStr">
         <is>
-          <t>$66,100.00</t>
+          <t>$26,600.00</t>
         </is>
       </c>
       <c r="AO24" s="11" t="n"/>
       <c r="AP24" s="11" t="inlineStr">
         <is>
-          <t>$29.62</t>
+          <t>$11.92</t>
         </is>
       </c>
       <c r="AQ24" s="11" t="inlineStr">
         <is>
-          <t>$44.43</t>
+          <t>$17.88</t>
         </is>
       </c>
       <c r="AR24" s="11" t="inlineStr">
@@ -55753,7 +55753,7 @@
       </c>
       <c r="AS24" s="11" t="inlineStr">
         <is>
-          <t>$2,600.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="AT24" s="11" t="inlineStr">
@@ -55763,7 +55763,7 @@
       </c>
       <c r="AU24" s="11" t="inlineStr">
         <is>
-          <t>$64,200.00</t>
+          <t>$25,800.00</t>
         </is>
       </c>
       <c r="AV24" s="11" t="inlineStr">
@@ -55831,7 +55831,7 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>01/17/1970</t>
+          <t>11/19/2000</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
@@ -55856,7 +55856,7 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>39-3092</t>
+          <t>11-9081</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
@@ -55866,7 +55866,7 @@
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>Costume Attendants</t>
+          <t>Lodging Managers</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
@@ -55876,7 +55876,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>09/27/2022</t>
+          <t>06/12/2024</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -55904,12 +55904,12 @@
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="inlineStr">
         <is>
-          <t>$16.11</t>
+          <t>$15.82</t>
         </is>
       </c>
       <c r="T25" s="13" t="inlineStr">
         <is>
-          <t>$24.16</t>
+          <t>$23.73</t>
         </is>
       </c>
       <c r="U25" s="11" t="inlineStr">
@@ -55939,18 +55939,18 @@
       </c>
       <c r="Z25" s="11" t="inlineStr">
         <is>
-          <t>$34,900.00</t>
+          <t>$34,300.00</t>
         </is>
       </c>
       <c r="AA25" s="11" t="n"/>
       <c r="AB25" s="11" t="inlineStr">
         <is>
-          <t>$15.62</t>
+          <t>$15.38</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>$23.43</t>
+          <t>$23.07</t>
         </is>
       </c>
       <c r="AD25" s="11" t="inlineStr">
@@ -55960,7 +55960,7 @@
       </c>
       <c r="AE25" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AF25" s="11" t="inlineStr">
@@ -55970,18 +55970,18 @@
       </c>
       <c r="AG25" s="11" t="inlineStr">
         <is>
-          <t>$33,900.00</t>
+          <t>$33,300.00</t>
         </is>
       </c>
       <c r="AH25" s="11" t="n"/>
       <c r="AI25" s="11" t="inlineStr">
         <is>
-          <t>$15.19</t>
+          <t>$14.90</t>
         </is>
       </c>
       <c r="AJ25" s="11" t="inlineStr">
         <is>
-          <t>$22.79</t>
+          <t>$22.35</t>
         </is>
       </c>
       <c r="AK25" s="11" t="inlineStr">
@@ -56001,18 +56001,18 @@
       </c>
       <c r="AN25" s="11" t="inlineStr">
         <is>
-          <t>$32,900.00</t>
+          <t>$32,300.00</t>
         </is>
       </c>
       <c r="AO25" s="11" t="n"/>
       <c r="AP25" s="11" t="inlineStr">
         <is>
-          <t>$14.71</t>
+          <t>$14.47</t>
         </is>
       </c>
       <c r="AQ25" s="11" t="inlineStr">
         <is>
-          <t>$22.07</t>
+          <t>$21.71</t>
         </is>
       </c>
       <c r="AR25" s="11" t="inlineStr">
@@ -56032,7 +56032,7 @@
       </c>
       <c r="AU25" s="11" t="inlineStr">
         <is>
-          <t>$31,900.00</t>
+          <t>$31,400.00</t>
         </is>
       </c>
       <c r="AV25" s="11" t="inlineStr">
@@ -56100,12 +56100,12 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>03/23/1980</t>
+          <t>08/08/1997</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
@@ -56125,7 +56125,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>11-9081</t>
+          <t>43-5061</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
@@ -56135,7 +56135,7 @@
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>Lodging Managers</t>
+          <t>Production, Planning, and Expediting Clerks</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
@@ -56145,7 +56145,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>02/17/2025</t>
+          <t>01/24/2022</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56173,12 +56173,12 @@
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="inlineStr">
         <is>
-          <t>$17.93</t>
+          <t>$15.82</t>
         </is>
       </c>
       <c r="T26" s="13" t="inlineStr">
         <is>
-          <t>$26.89</t>
+          <t>$23.73</t>
         </is>
       </c>
       <c r="U26" s="11" t="inlineStr">
@@ -56198,7 +56198,7 @@
       </c>
       <c r="X26" s="11" t="inlineStr">
         <is>
-          <t>$1,600.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="Y26" s="11" t="inlineStr">
@@ -56208,18 +56208,18 @@
       </c>
       <c r="Z26" s="11" t="inlineStr">
         <is>
-          <t>$38,900.00</t>
+          <t>$34,300.00</t>
         </is>
       </c>
       <c r="AA26" s="11" t="n"/>
       <c r="AB26" s="11" t="inlineStr">
         <is>
-          <t>$17.45</t>
+          <t>$15.38</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>$26.17</t>
+          <t>$23.07</t>
         </is>
       </c>
       <c r="AD26" s="11" t="inlineStr">
@@ -56229,7 +56229,7 @@
       </c>
       <c r="AE26" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AF26" s="11" t="inlineStr">
@@ -56239,18 +56239,18 @@
       </c>
       <c r="AG26" s="11" t="inlineStr">
         <is>
-          <t>$37,800.00</t>
+          <t>$33,300.00</t>
         </is>
       </c>
       <c r="AH26" s="11" t="n"/>
       <c r="AI26" s="11" t="inlineStr">
         <is>
-          <t>$16.92</t>
+          <t>$14.90</t>
         </is>
       </c>
       <c r="AJ26" s="11" t="inlineStr">
         <is>
-          <t>$25.38</t>
+          <t>$22.35</t>
         </is>
       </c>
       <c r="AK26" s="11" t="inlineStr">
@@ -56260,7 +56260,7 @@
       </c>
       <c r="AL26" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AM26" s="11" t="inlineStr">
@@ -56270,18 +56270,18 @@
       </c>
       <c r="AN26" s="11" t="inlineStr">
         <is>
-          <t>$36,700.00</t>
+          <t>$32,300.00</t>
         </is>
       </c>
       <c r="AO26" s="11" t="n"/>
       <c r="AP26" s="11" t="inlineStr">
         <is>
-          <t>$16.44</t>
+          <t>$14.47</t>
         </is>
       </c>
       <c r="AQ26" s="11" t="inlineStr">
         <is>
-          <t>$24.66</t>
+          <t>$21.71</t>
         </is>
       </c>
       <c r="AR26" s="11" t="inlineStr">
@@ -56291,7 +56291,7 @@
       </c>
       <c r="AS26" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AT26" s="11" t="inlineStr">
@@ -56301,7 +56301,7 @@
       </c>
       <c r="AU26" s="11" t="inlineStr">
         <is>
-          <t>$35,600.00</t>
+          <t>$31,400.00</t>
         </is>
       </c>
       <c r="AV26" s="11" t="inlineStr">
@@ -56369,7 +56369,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>12/28/1977</t>
+          <t>02/18/1979</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
@@ -56394,7 +56394,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>43-6011</t>
+          <t>49-3042</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
@@ -56404,7 +56404,7 @@
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>Executive Secretaries and Executive Administrative Assistants</t>
+          <t>Mobile Heavy Equipment Mechanics, Except Engines</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
@@ -56414,7 +56414,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>06/12/2024</t>
+          <t>07/08/2013</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56447,7 +56447,7 @@
       </c>
       <c r="T27" s="13" t="inlineStr">
         <is>
-          <t>$26.54</t>
+          <t>$23.73</t>
         </is>
       </c>
       <c r="U27" s="11" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="X27" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="Y27" s="11" t="inlineStr">
@@ -56483,12 +56483,12 @@
       <c r="AA27" s="11" t="n"/>
       <c r="AB27" s="11" t="inlineStr">
         <is>
-          <t>$17.16</t>
+          <t>$15.38</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>$25.74</t>
+          <t>$23.07</t>
         </is>
       </c>
       <c r="AD27" s="11" t="inlineStr">
@@ -56498,7 +56498,7 @@
       </c>
       <c r="AE27" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AF27" s="11" t="inlineStr">
@@ -56508,18 +56508,18 @@
       </c>
       <c r="AG27" s="11" t="inlineStr">
         <is>
-          <t>$37,200.00</t>
+          <t>$33,300.00</t>
         </is>
       </c>
       <c r="AH27" s="11" t="n"/>
       <c r="AI27" s="11" t="inlineStr">
         <is>
-          <t>$16.68</t>
+          <t>$14.90</t>
         </is>
       </c>
       <c r="AJ27" s="11" t="inlineStr">
         <is>
-          <t>$25.02</t>
+          <t>$22.35</t>
         </is>
       </c>
       <c r="AK27" s="11" t="inlineStr">
@@ -56529,7 +56529,7 @@
       </c>
       <c r="AL27" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AM27" s="11" t="inlineStr">
@@ -56539,18 +56539,18 @@
       </c>
       <c r="AN27" s="11" t="inlineStr">
         <is>
-          <t>$36,100.00</t>
+          <t>$32,300.00</t>
         </is>
       </c>
       <c r="AO27" s="11" t="n"/>
       <c r="AP27" s="11" t="inlineStr">
         <is>
-          <t>$16.15</t>
+          <t>$14.47</t>
         </is>
       </c>
       <c r="AQ27" s="11" t="inlineStr">
         <is>
-          <t>$24.22</t>
+          <t>$21.71</t>
         </is>
       </c>
       <c r="AR27" s="11" t="inlineStr">
@@ -56560,7 +56560,7 @@
       </c>
       <c r="AS27" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="AT27" s="11" t="inlineStr">
@@ -56570,7 +56570,7 @@
       </c>
       <c r="AU27" s="11" t="inlineStr">
         <is>
-          <t>$35,000.00</t>
+          <t>$31,400.00</t>
         </is>
       </c>
       <c r="AV27" s="11" t="inlineStr">
@@ -56638,7 +56638,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>02/10/1975</t>
+          <t>10/18/1967</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
@@ -56663,7 +56663,7 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>49-9069</t>
+          <t>53-7065</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
@@ -56673,7 +56673,7 @@
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>Precision Instrument and Equipment Repairers, All Other</t>
+          <t>Stockers and Order Fillers</t>
         </is>
       </c>
       <c r="J28" s="14" t="inlineStr">
@@ -56683,7 +56683,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>11/24/2017</t>
+          <t>05/28/2019</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56711,12 +56711,12 @@
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="inlineStr">
         <is>
-          <t>$14.09</t>
+          <t>$11.44</t>
         </is>
       </c>
       <c r="T28" s="13" t="inlineStr">
         <is>
-          <t>$21.13</t>
+          <t>$17.16</t>
         </is>
       </c>
       <c r="U28" s="11" t="inlineStr">
@@ -56736,7 +56736,7 @@
       </c>
       <c r="X28" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="Y28" s="11" t="inlineStr">
@@ -56746,18 +56746,18 @@
       </c>
       <c r="Z28" s="11" t="inlineStr">
         <is>
-          <t>$30,500.00</t>
+          <t>$24,800.00</t>
         </is>
       </c>
       <c r="AA28" s="11" t="n"/>
       <c r="AB28" s="11" t="inlineStr">
         <is>
-          <t>$13.65</t>
+          <t>$11.11</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>$20.48</t>
+          <t>$16.66</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
@@ -56767,7 +56767,7 @@
       </c>
       <c r="AE28" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="AF28" s="11" t="inlineStr">
@@ -56777,18 +56777,18 @@
       </c>
       <c r="AG28" s="11" t="inlineStr">
         <is>
-          <t>$29,600.00</t>
+          <t>$24,100.00</t>
         </is>
       </c>
       <c r="AH28" s="11" t="n"/>
       <c r="AI28" s="11" t="inlineStr">
         <is>
-          <t>$13.27</t>
+          <t>$10.82</t>
         </is>
       </c>
       <c r="AJ28" s="11" t="inlineStr">
         <is>
-          <t>$19.91</t>
+          <t>$16.23</t>
         </is>
       </c>
       <c r="AK28" s="11" t="inlineStr">
@@ -56798,7 +56798,7 @@
       </c>
       <c r="AL28" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="AM28" s="11" t="inlineStr">
@@ -56808,18 +56808,18 @@
       </c>
       <c r="AN28" s="11" t="inlineStr">
         <is>
-          <t>$28,700.00</t>
+          <t>$23,400.00</t>
         </is>
       </c>
       <c r="AO28" s="11" t="n"/>
       <c r="AP28" s="11" t="inlineStr">
         <is>
-          <t>$12.88</t>
+          <t>$10.48</t>
         </is>
       </c>
       <c r="AQ28" s="11" t="inlineStr">
         <is>
-          <t>$19.32</t>
+          <t>$15.72</t>
         </is>
       </c>
       <c r="AR28" s="11" t="inlineStr">
@@ -56829,7 +56829,7 @@
       </c>
       <c r="AS28" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="AT28" s="11" t="inlineStr">
@@ -56839,7 +56839,7 @@
       </c>
       <c r="AU28" s="11" t="inlineStr">
         <is>
-          <t>$27,900.00</t>
+          <t>$22,700.00</t>
         </is>
       </c>
       <c r="AV28" s="11" t="inlineStr">
@@ -56907,7 +56907,7 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>02/18/1995</t>
+          <t>12/04/1981</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
@@ -56932,7 +56932,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>53-7065</t>
+          <t>31-2011</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
@@ -56942,7 +56942,7 @@
       </c>
       <c r="I29" s="14" t="inlineStr">
         <is>
-          <t>Stockers and Order Fillers</t>
+          <t>Occupational Therapy Assistants</t>
         </is>
       </c>
       <c r="J29" s="14" t="inlineStr">
@@ -56952,7 +56952,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>01/02/2017</t>
+          <t>06/17/2019</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -56980,12 +56980,12 @@
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="inlineStr">
         <is>
-          <t>$11.44</t>
+          <t>$17.69</t>
         </is>
       </c>
       <c r="T29" s="13" t="inlineStr">
         <is>
-          <t>$17.16</t>
+          <t>$26.54</t>
         </is>
       </c>
       <c r="U29" s="11" t="inlineStr">
@@ -57005,7 +57005,7 @@
       </c>
       <c r="X29" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="Y29" s="11" t="inlineStr">
@@ -57015,18 +57015,18 @@
       </c>
       <c r="Z29" s="11" t="inlineStr">
         <is>
-          <t>$24,800.00</t>
+          <t>$38,300.00</t>
         </is>
       </c>
       <c r="AA29" s="11" t="n"/>
       <c r="AB29" s="11" t="inlineStr">
         <is>
-          <t>$11.11</t>
+          <t>$17.16</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>$16.66</t>
+          <t>$25.74</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
@@ -57036,7 +57036,7 @@
       </c>
       <c r="AE29" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="AF29" s="11" t="inlineStr">
@@ -57046,18 +57046,18 @@
       </c>
       <c r="AG29" s="11" t="inlineStr">
         <is>
-          <t>$24,100.00</t>
+          <t>$37,200.00</t>
         </is>
       </c>
       <c r="AH29" s="11" t="n"/>
       <c r="AI29" s="11" t="inlineStr">
         <is>
-          <t>$10.82</t>
+          <t>$16.68</t>
         </is>
       </c>
       <c r="AJ29" s="11" t="inlineStr">
         <is>
-          <t>$16.23</t>
+          <t>$25.02</t>
         </is>
       </c>
       <c r="AK29" s="11" t="inlineStr">
@@ -57067,7 +57067,7 @@
       </c>
       <c r="AL29" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="AM29" s="11" t="inlineStr">
@@ -57077,18 +57077,18 @@
       </c>
       <c r="AN29" s="11" t="inlineStr">
         <is>
-          <t>$23,400.00</t>
+          <t>$36,100.00</t>
         </is>
       </c>
       <c r="AO29" s="11" t="n"/>
       <c r="AP29" s="11" t="inlineStr">
         <is>
-          <t>$10.48</t>
+          <t>$16.15</t>
         </is>
       </c>
       <c r="AQ29" s="11" t="inlineStr">
         <is>
-          <t>$15.72</t>
+          <t>$24.22</t>
         </is>
       </c>
       <c r="AR29" s="11" t="inlineStr">
@@ -57098,7 +57098,7 @@
       </c>
       <c r="AS29" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="AT29" s="11" t="inlineStr">
@@ -57108,7 +57108,7 @@
       </c>
       <c r="AU29" s="11" t="inlineStr">
         <is>
-          <t>$22,700.00</t>
+          <t>$35,000.00</t>
         </is>
       </c>
       <c r="AV29" s="11" t="inlineStr">
@@ -57176,12 +57176,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>11/03/1984</t>
+          <t>02/06/1991</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57201,7 +57201,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>29-1181</t>
+          <t>15-1299</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
@@ -57211,7 +57211,7 @@
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>Audiologists</t>
+          <t>Information Technology Project Managers</t>
         </is>
       </c>
       <c r="J30" s="14" t="inlineStr">
@@ -57221,7 +57221,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>11/25/2024</t>
+          <t>02/25/2021</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57249,12 +57249,12 @@
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="inlineStr">
         <is>
-          <t>$27.69</t>
+          <t>$19.09</t>
         </is>
       </c>
       <c r="T30" s="13" t="inlineStr">
         <is>
-          <t>$41.54</t>
+          <t>$28.63</t>
         </is>
       </c>
       <c r="U30" s="11" t="inlineStr">
@@ -57274,7 +57274,7 @@
       </c>
       <c r="X30" s="11" t="inlineStr">
         <is>
-          <t>$2,400.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="Y30" s="11" t="inlineStr">
@@ -57284,18 +57284,18 @@
       </c>
       <c r="Z30" s="11" t="inlineStr">
         <is>
-          <t>$60,000.00</t>
+          <t>$41,400.00</t>
         </is>
       </c>
       <c r="AA30" s="11" t="n"/>
       <c r="AB30" s="11" t="inlineStr">
         <is>
-          <t>$26.92</t>
+          <t>$18.56</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>$40.38</t>
+          <t>$27.84</t>
         </is>
       </c>
       <c r="AD30" s="11" t="inlineStr">
@@ -57305,7 +57305,7 @@
       </c>
       <c r="AE30" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AF30" s="11" t="inlineStr">
@@ -57315,18 +57315,18 @@
       </c>
       <c r="AG30" s="11" t="inlineStr">
         <is>
-          <t>$58,300.00</t>
+          <t>$40,200.00</t>
         </is>
       </c>
       <c r="AH30" s="11" t="n"/>
       <c r="AI30" s="11" t="inlineStr">
         <is>
-          <t>$26.11</t>
+          <t>$17.98</t>
         </is>
       </c>
       <c r="AJ30" s="11" t="inlineStr">
         <is>
-          <t>$39.16</t>
+          <t>$26.97</t>
         </is>
       </c>
       <c r="AK30" s="11" t="inlineStr">
@@ -57336,7 +57336,7 @@
       </c>
       <c r="AL30" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AM30" s="11" t="inlineStr">
@@ -57346,18 +57346,18 @@
       </c>
       <c r="AN30" s="11" t="inlineStr">
         <is>
-          <t>$56,600.00</t>
+          <t>$39,000.00</t>
         </is>
       </c>
       <c r="AO30" s="11" t="n"/>
       <c r="AP30" s="11" t="inlineStr">
         <is>
-          <t>$25.38</t>
+          <t>$17.50</t>
         </is>
       </c>
       <c r="AQ30" s="11" t="inlineStr">
         <is>
-          <t>$38.07</t>
+          <t>$26.25</t>
         </is>
       </c>
       <c r="AR30" s="11" t="inlineStr">
@@ -57367,7 +57367,7 @@
       </c>
       <c r="AS30" s="11" t="inlineStr">
         <is>
-          <t>$2,200.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="AT30" s="11" t="inlineStr">
@@ -57377,7 +57377,7 @@
       </c>
       <c r="AU30" s="11" t="inlineStr">
         <is>
-          <t>$55,000.00</t>
+          <t>$37,900.00</t>
         </is>
       </c>
       <c r="AV30" s="11" t="inlineStr">
@@ -57445,12 +57445,12 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>03/15/2000</t>
+          <t>10/10/1999</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -57470,7 +57470,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>15-1299</t>
+          <t>47-4011</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -57480,7 +57480,7 @@
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>Penetration Testers</t>
+          <t>Energy Auditors</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
@@ -57490,7 +57490,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>03/22/2022</t>
+          <t>06/25/2018</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57518,12 +57518,12 @@
       <c r="R31" s="14" t="n"/>
       <c r="S31" s="14" t="inlineStr">
         <is>
-          <t>$26.83</t>
+          <t>$22.84</t>
         </is>
       </c>
       <c r="T31" s="13" t="inlineStr">
         <is>
-          <t>$40.24</t>
+          <t>$34.26</t>
         </is>
       </c>
       <c r="U31" s="11" t="inlineStr">
@@ -57543,7 +57543,7 @@
       </c>
       <c r="X31" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$2,000.00</t>
         </is>
       </c>
       <c r="Y31" s="11" t="inlineStr">
@@ -57553,18 +57553,18 @@
       </c>
       <c r="Z31" s="11" t="inlineStr">
         <is>
-          <t>$58,100.00</t>
+          <t>$49,500.00</t>
         </is>
       </c>
       <c r="AA31" s="11" t="n"/>
       <c r="AB31" s="11" t="inlineStr">
         <is>
-          <t>$26.01</t>
+          <t>$22.21</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>$39.02</t>
+          <t>$33.31</t>
         </is>
       </c>
       <c r="AD31" s="11" t="inlineStr">
@@ -57574,7 +57574,7 @@
       </c>
       <c r="AE31" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$1,900.00</t>
         </is>
       </c>
       <c r="AF31" s="11" t="inlineStr">
@@ -57584,18 +57584,18 @@
       </c>
       <c r="AG31" s="11" t="inlineStr">
         <is>
-          <t>$56,400.00</t>
+          <t>$48,100.00</t>
         </is>
       </c>
       <c r="AH31" s="11" t="n"/>
       <c r="AI31" s="11" t="inlineStr">
         <is>
-          <t>$25.29</t>
+          <t>$21.54</t>
         </is>
       </c>
       <c r="AJ31" s="11" t="inlineStr">
         <is>
-          <t>$37.94</t>
+          <t>$32.31</t>
         </is>
       </c>
       <c r="AK31" s="11" t="inlineStr">
@@ -57605,7 +57605,7 @@
       </c>
       <c r="AL31" s="11" t="inlineStr">
         <is>
-          <t>$2,200.00</t>
+          <t>$1,900.00</t>
         </is>
       </c>
       <c r="AM31" s="11" t="inlineStr">
@@ -57615,18 +57615,18 @@
       </c>
       <c r="AN31" s="11" t="inlineStr">
         <is>
-          <t>$54,800.00</t>
+          <t>$46,700.00</t>
         </is>
       </c>
       <c r="AO31" s="11" t="n"/>
       <c r="AP31" s="11" t="inlineStr">
         <is>
-          <t>$24.57</t>
+          <t>$20.91</t>
         </is>
       </c>
       <c r="AQ31" s="11" t="inlineStr">
         <is>
-          <t>$36.86</t>
+          <t>$31.37</t>
         </is>
       </c>
       <c r="AR31" s="11" t="inlineStr">
@@ -57636,7 +57636,7 @@
       </c>
       <c r="AS31" s="11" t="inlineStr">
         <is>
-          <t>$2,100.00</t>
+          <t>$1,800.00</t>
         </is>
       </c>
       <c r="AT31" s="11" t="inlineStr">
@@ -57646,7 +57646,7 @@
       </c>
       <c r="AU31" s="11" t="inlineStr">
         <is>
-          <t>$53,200.00</t>
+          <t>$45,300.00</t>
         </is>
       </c>
       <c r="AV31" s="11" t="inlineStr">
@@ -57714,12 +57714,12 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>03/19/1972</t>
+          <t>10/10/1979</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -57739,7 +57739,7 @@
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>53-3053</t>
+          <t>53-5031</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
@@ -57749,7 +57749,7 @@
       </c>
       <c r="I32" s="14" t="inlineStr">
         <is>
-          <t>Shuttle Drivers and Chauffeurs</t>
+          <t>Ship Engineers</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
@@ -57759,7 +57759,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>08/10/2016</t>
+          <t>06/20/2023</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57787,12 +57787,12 @@
       <c r="R32" s="14" t="n"/>
       <c r="S32" s="14" t="inlineStr">
         <is>
-          <t>$12.69</t>
+          <t>$28.80</t>
         </is>
       </c>
       <c r="T32" s="13" t="inlineStr">
         <is>
-          <t>$19.04</t>
+          <t>$43.20</t>
         </is>
       </c>
       <c r="U32" s="11" t="inlineStr">
@@ -57812,7 +57812,7 @@
       </c>
       <c r="X32" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$2,500.00</t>
         </is>
       </c>
       <c r="Y32" s="11" t="inlineStr">
@@ -57822,18 +57822,18 @@
       </c>
       <c r="Z32" s="11" t="inlineStr">
         <is>
-          <t>$27,500.00</t>
+          <t>$62,400.00</t>
         </is>
       </c>
       <c r="AA32" s="11" t="n"/>
       <c r="AB32" s="11" t="inlineStr">
         <is>
-          <t>$12.31</t>
+          <t>$27.98</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>$18.46</t>
+          <t>$41.97</t>
         </is>
       </c>
       <c r="AD32" s="11" t="inlineStr">
@@ -57843,7 +57843,7 @@
       </c>
       <c r="AE32" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$2,400.00</t>
         </is>
       </c>
       <c r="AF32" s="11" t="inlineStr">
@@ -57853,18 +57853,18 @@
       </c>
       <c r="AG32" s="11" t="inlineStr">
         <is>
-          <t>$26,700.00</t>
+          <t>$60,600.00</t>
         </is>
       </c>
       <c r="AH32" s="11" t="n"/>
       <c r="AI32" s="11" t="inlineStr">
         <is>
-          <t>$11.97</t>
+          <t>$27.12</t>
         </is>
       </c>
       <c r="AJ32" s="11" t="inlineStr">
         <is>
-          <t>$17.96</t>
+          <t>$40.68</t>
         </is>
       </c>
       <c r="AK32" s="11" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="AL32" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$2,400.00</t>
         </is>
       </c>
       <c r="AM32" s="11" t="inlineStr">
@@ -57884,18 +57884,18 @@
       </c>
       <c r="AN32" s="11" t="inlineStr">
         <is>
-          <t>$25,900.00</t>
+          <t>$58,800.00</t>
         </is>
       </c>
       <c r="AO32" s="11" t="n"/>
       <c r="AP32" s="11" t="inlineStr">
         <is>
-          <t>$11.59</t>
+          <t>$26.35</t>
         </is>
       </c>
       <c r="AQ32" s="11" t="inlineStr">
         <is>
-          <t>$17.38</t>
+          <t>$39.53</t>
         </is>
       </c>
       <c r="AR32" s="11" t="inlineStr">
@@ -57905,7 +57905,7 @@
       </c>
       <c r="AS32" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$2,300.00</t>
         </is>
       </c>
       <c r="AT32" s="11" t="inlineStr">
@@ -57915,7 +57915,7 @@
       </c>
       <c r="AU32" s="11" t="inlineStr">
         <is>
-          <t>$25,100.00</t>
+          <t>$57,100.00</t>
         </is>
       </c>
       <c r="AV32" s="11" t="inlineStr">
@@ -57983,12 +57983,12 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>10/02/1991</t>
+          <t>11/19/1992</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D33" s="21" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>33-9011</t>
+          <t>29-1124</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -58018,7 +58018,7 @@
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>Animal Control Workers</t>
+          <t>Radiation Therapists</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
@@ -58028,7 +58028,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>04/17/2018</t>
+          <t>06/13/2020</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58056,12 +58056,12 @@
       <c r="R33" s="14" t="n"/>
       <c r="S33" s="14" t="inlineStr">
         <is>
-          <t>$10.38</t>
+          <t>$27.74</t>
         </is>
       </c>
       <c r="T33" s="13" t="inlineStr">
         <is>
-          <t>$15.57</t>
+          <t>$41.61</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -58081,7 +58081,7 @@
       </c>
       <c r="X33" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$2,400.00</t>
         </is>
       </c>
       <c r="Y33" s="11" t="inlineStr">
@@ -58091,18 +58091,18 @@
       </c>
       <c r="Z33" s="11" t="inlineStr">
         <is>
-          <t>$22,500.00</t>
+          <t>$60,100.00</t>
         </is>
       </c>
       <c r="AA33" s="11" t="n"/>
       <c r="AB33" s="11" t="inlineStr">
         <is>
-          <t>$10.05</t>
+          <t>$26.92</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>$15.08</t>
+          <t>$40.38</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
@@ -58112,7 +58112,7 @@
       </c>
       <c r="AE33" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$2,300.00</t>
         </is>
       </c>
       <c r="AF33" s="11" t="inlineStr">
@@ -58122,18 +58122,18 @@
       </c>
       <c r="AG33" s="11" t="inlineStr">
         <is>
-          <t>$21,800.00</t>
+          <t>$58,300.00</t>
         </is>
       </c>
       <c r="AH33" s="11" t="n"/>
       <c r="AI33" s="11" t="inlineStr">
         <is>
-          <t>$9.81</t>
+          <t>$26.11</t>
         </is>
       </c>
       <c r="AJ33" s="11" t="inlineStr">
         <is>
-          <t>$14.71</t>
+          <t>$39.16</t>
         </is>
       </c>
       <c r="AK33" s="11" t="inlineStr">
@@ -58143,7 +58143,7 @@
       </c>
       <c r="AL33" s="11" t="inlineStr">
         <is>
-          <t>$800.00</t>
+          <t>$2,300.00</t>
         </is>
       </c>
       <c r="AM33" s="11" t="inlineStr">
@@ -58153,18 +58153,18 @@
       </c>
       <c r="AN33" s="11" t="inlineStr">
         <is>
-          <t>$21,200.00</t>
+          <t>$56,600.00</t>
         </is>
       </c>
       <c r="AO33" s="11" t="n"/>
       <c r="AP33" s="11" t="inlineStr">
         <is>
-          <t>$9.52</t>
+          <t>$25.38</t>
         </is>
       </c>
       <c r="AQ33" s="11" t="inlineStr">
         <is>
-          <t>$14.28</t>
+          <t>$38.07</t>
         </is>
       </c>
       <c r="AR33" s="11" t="inlineStr">
@@ -58174,7 +58174,7 @@
       </c>
       <c r="AS33" s="11" t="inlineStr">
         <is>
-          <t>$800.00</t>
+          <t>$2,200.00</t>
         </is>
       </c>
       <c r="AT33" s="11" t="inlineStr">
@@ -58184,7 +58184,7 @@
       </c>
       <c r="AU33" s="11" t="inlineStr">
         <is>
-          <t>$20,600.00</t>
+          <t>$55,000.00</t>
         </is>
       </c>
       <c r="AV33" s="11" t="inlineStr">
@@ -58252,12 +58252,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>05/09/1990</t>
+          <t>02/26/1971</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
@@ -58277,7 +58277,7 @@
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>49-3092</t>
+          <t>31-1132</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
@@ -58287,7 +58287,7 @@
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>Recreational Vehicle Service Technicians</t>
+          <t>Orderlies</t>
         </is>
       </c>
       <c r="J34" s="14" t="inlineStr">
@@ -58297,7 +58297,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>03/18/2014</t>
+          <t>06/06/2013</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58325,12 +58325,12 @@
       <c r="R34" s="14" t="n"/>
       <c r="S34" s="14" t="inlineStr">
         <is>
-          <t>$14.04</t>
+          <t>$13.27</t>
         </is>
       </c>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>$21.06</t>
+          <t>$19.91</t>
         </is>
       </c>
       <c r="U34" s="11" t="inlineStr">
@@ -58360,18 +58360,18 @@
       </c>
       <c r="Z34" s="11" t="inlineStr">
         <is>
-          <t>$30,400.00</t>
+          <t>$28,800.00</t>
         </is>
       </c>
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="11" t="inlineStr">
         <is>
-          <t>$13.61</t>
+          <t>$12.93</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>$20.41</t>
+          <t>$19.39</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
@@ -58381,7 +58381,7 @@
       </c>
       <c r="AE34" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AF34" s="11" t="inlineStr">
@@ -58391,18 +58391,18 @@
       </c>
       <c r="AG34" s="11" t="inlineStr">
         <is>
-          <t>$29,500.00</t>
+          <t>$28,000.00</t>
         </is>
       </c>
       <c r="AH34" s="11" t="n"/>
       <c r="AI34" s="11" t="inlineStr">
         <is>
-          <t>$13.22</t>
+          <t>$12.55</t>
         </is>
       </c>
       <c r="AJ34" s="11" t="inlineStr">
         <is>
-          <t>$19.83</t>
+          <t>$18.83</t>
         </is>
       </c>
       <c r="AK34" s="11" t="inlineStr">
@@ -58422,18 +58422,18 @@
       </c>
       <c r="AN34" s="11" t="inlineStr">
         <is>
-          <t>$28,600.00</t>
+          <t>$27,200.00</t>
         </is>
       </c>
       <c r="AO34" s="11" t="n"/>
       <c r="AP34" s="11" t="inlineStr">
         <is>
-          <t>$12.84</t>
+          <t>$12.16</t>
         </is>
       </c>
       <c r="AQ34" s="11" t="inlineStr">
         <is>
-          <t>$19.26</t>
+          <t>$18.24</t>
         </is>
       </c>
       <c r="AR34" s="11" t="inlineStr">
@@ -58453,7 +58453,7 @@
       </c>
       <c r="AU34" s="11" t="inlineStr">
         <is>
-          <t>$27,800.00</t>
+          <t>$26,400.00</t>
         </is>
       </c>
       <c r="AV34" s="11" t="inlineStr">
@@ -58521,7 +58521,7 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>07/07/1980</t>
+          <t>11/07/1996</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
@@ -58546,7 +58546,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>29-1029</t>
+          <t>51-9011</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
@@ -58556,7 +58556,7 @@
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>Dentists, All Other Specialists</t>
+          <t>Chemical Equipment Operators and Tenders</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
@@ -58566,7 +58566,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>05/13/2020</t>
+          <t>04/27/2022</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -58594,12 +58594,12 @@
       <c r="R35" s="14" t="n"/>
       <c r="S35" s="14" t="inlineStr">
         <is>
-          <t>$63.03</t>
+          <t>$13.22</t>
         </is>
       </c>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>$94.55</t>
+          <t>$19.83</t>
         </is>
       </c>
       <c r="U35" s="11" t="inlineStr">
@@ -58619,7 +58619,7 @@
       </c>
       <c r="X35" s="11" t="inlineStr">
         <is>
-          <t>$5,500.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="Y35" s="11" t="inlineStr">
@@ -58629,18 +58629,18 @@
       </c>
       <c r="Z35" s="11" t="inlineStr">
         <is>
-          <t>$136,600.00</t>
+          <t>$28,600.00</t>
         </is>
       </c>
       <c r="AA35" s="11" t="n"/>
       <c r="AB35" s="11" t="inlineStr">
         <is>
-          <t>$61.20</t>
+          <t>$12.84</t>
         </is>
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>$91.80</t>
+          <t>$19.26</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
@@ -58650,7 +58650,7 @@
       </c>
       <c r="AE35" s="11" t="inlineStr">
         <is>
-          <t>$5,300.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AF35" s="11" t="inlineStr">
@@ -58660,18 +58660,18 @@
       </c>
       <c r="AG35" s="11" t="inlineStr">
         <is>
-          <t>$132,600.00</t>
+          <t>$27,800.00</t>
         </is>
       </c>
       <c r="AH35" s="11" t="n"/>
       <c r="AI35" s="11" t="inlineStr">
         <is>
-          <t>$59.42</t>
+          <t>$12.45</t>
         </is>
       </c>
       <c r="AJ35" s="11" t="inlineStr">
         <is>
-          <t>$89.13</t>
+          <t>$18.67</t>
         </is>
       </c>
       <c r="AK35" s="11" t="inlineStr">
@@ -58681,7 +58681,7 @@
       </c>
       <c r="AL35" s="11" t="inlineStr">
         <is>
-          <t>$5,100.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AM35" s="11" t="inlineStr">
@@ -58691,18 +58691,18 @@
       </c>
       <c r="AN35" s="11" t="inlineStr">
         <is>
-          <t>$128,700.00</t>
+          <t>$27,000.00</t>
         </is>
       </c>
       <c r="AO35" s="11" t="n"/>
       <c r="AP35" s="11" t="inlineStr">
         <is>
-          <t>$57.69</t>
+          <t>$12.12</t>
         </is>
       </c>
       <c r="AQ35" s="11" t="inlineStr">
         <is>
-          <t>$86.53</t>
+          <t>$18.18</t>
         </is>
       </c>
       <c r="AR35" s="11" t="inlineStr">
@@ -58712,7 +58712,7 @@
       </c>
       <c r="AS35" s="11" t="inlineStr">
         <is>
-          <t>$5,000.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="AT35" s="11" t="inlineStr">
@@ -58722,7 +58722,7 @@
       </c>
       <c r="AU35" s="11" t="inlineStr">
         <is>
-          <t>$125,000.00</t>
+          <t>$26,200.00</t>
         </is>
       </c>
       <c r="AV35" s="11" t="inlineStr">
@@ -65462,7 +65462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-20 18:20 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-20 19:47 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(test-plan): M-25 covers SOC derivation beyond the happy path
E28 already proved a clean O*NET title resolves. M-25 adds the cases a
real census actually produces, each taking a different branch of
match_soc: no title at all, an invented title, an ambiguous one-word
title, and a supplied code that contradicts the role.

The expected result names what should happen in each - unmatched rather
than a placeholder, routed to review rather than forced onto the nearest
occupation, a rival surfaced with its confidence, and a census code
winning while its disagreement with the title is still flagged.

Also re-syncs the downloadable fixtures so edge_ingestion.xlsx carries
E29-E32.

Verified on a scratch Postgres 16: applies after the earlier case
migrations, 25 cases total, re-running does not duplicate.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53146,7 +53146,7 @@
       </c>
       <c r="B9" s="43" t="inlineStr">
         <is>
-          <t>07/20/2026</t>
+          <t>07/21/2026</t>
         </is>
       </c>
       <c r="C9" s="43" t="n"/>
@@ -53940,12 +53940,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>09/21/1974</t>
+          <t>08/12/1981</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53985,7 +53985,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>06/04/2013</t>
+          <t>03/04/2013</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54209,7 +54209,7 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>08/12/1989</t>
+          <t>12/12/1997</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
@@ -54254,7 +54254,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>06/01/2021</t>
+          <t>05/26/2021</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54478,7 +54478,7 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>04/24/1997</t>
+          <t>08/24/1985</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
@@ -54523,7 +54523,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>12/06/2018</t>
+          <t>02/06/2019</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54763,12 +54763,12 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>03/19/1972</t>
+          <t>08/12/1997</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -54808,7 +54808,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>08/13/2020</t>
+          <t>03/03/2017</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55032,7 +55032,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>02/14/1995</t>
+          <t>12/04/1985</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -55077,7 +55077,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>07/23/2025</t>
+          <t>06/10/2012</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55566,12 +55566,12 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>08/04/1981</t>
+          <t>11/19/2000</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -55587,7 +55587,7 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>39-4031</t>
+          <t>51-9195</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
@@ -55597,7 +55597,7 @@
       </c>
       <c r="I24" s="14" t="inlineStr">
         <is>
-          <t>Morticians, Undertakers, and Funeral Arrangers</t>
+          <t>Glass Blowers, Molders, Benders, and Finishers</t>
         </is>
       </c>
       <c r="J24" s="14" t="inlineStr">
@@ -55607,7 +55607,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>07/12/2012</t>
+          <t>09/06/2020</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55635,12 +55635,12 @@
       <c r="R24" s="14" t="n"/>
       <c r="S24" s="14" t="inlineStr">
         <is>
-          <t>$13.03</t>
+          <t>$13.32</t>
         </is>
       </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
-          <t>$19.54</t>
+          <t>$19.98</t>
         </is>
       </c>
       <c r="U24" s="11" t="inlineStr">
@@ -55660,7 +55660,7 @@
       </c>
       <c r="X24" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$1,200.00</t>
         </is>
       </c>
       <c r="Y24" s="11" t="inlineStr">
@@ -55670,18 +55670,18 @@
       </c>
       <c r="Z24" s="11" t="inlineStr">
         <is>
-          <t>$28,200.00</t>
+          <t>$28,900.00</t>
         </is>
       </c>
       <c r="AA24" s="11" t="n"/>
       <c r="AB24" s="11" t="inlineStr">
         <is>
-          <t>$12.64</t>
+          <t>$12.98</t>
         </is>
       </c>
       <c r="AC24" s="11" t="inlineStr">
         <is>
-          <t>$18.96</t>
+          <t>$19.47</t>
         </is>
       </c>
       <c r="AD24" s="11" t="inlineStr">
@@ -55701,18 +55701,18 @@
       </c>
       <c r="AG24" s="11" t="inlineStr">
         <is>
-          <t>$27,400.00</t>
+          <t>$28,100.00</t>
         </is>
       </c>
       <c r="AH24" s="11" t="n"/>
       <c r="AI24" s="11" t="inlineStr">
         <is>
-          <t>$12.26</t>
+          <t>$12.60</t>
         </is>
       </c>
       <c r="AJ24" s="11" t="inlineStr">
         <is>
-          <t>$18.39</t>
+          <t>$18.90</t>
         </is>
       </c>
       <c r="AK24" s="11" t="inlineStr">
@@ -55732,18 +55732,18 @@
       </c>
       <c r="AN24" s="11" t="inlineStr">
         <is>
-          <t>$26,600.00</t>
+          <t>$27,300.00</t>
         </is>
       </c>
       <c r="AO24" s="11" t="n"/>
       <c r="AP24" s="11" t="inlineStr">
         <is>
-          <t>$11.92</t>
+          <t>$12.21</t>
         </is>
       </c>
       <c r="AQ24" s="11" t="inlineStr">
         <is>
-          <t>$17.88</t>
+          <t>$18.32</t>
         </is>
       </c>
       <c r="AR24" s="11" t="inlineStr">
@@ -55753,7 +55753,7 @@
       </c>
       <c r="AS24" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AT24" s="11" t="inlineStr">
@@ -55763,7 +55763,7 @@
       </c>
       <c r="AU24" s="11" t="inlineStr">
         <is>
-          <t>$25,800.00</t>
+          <t>$26,500.00</t>
         </is>
       </c>
       <c r="AV24" s="11" t="inlineStr">
@@ -55831,12 +55831,12 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>11/19/2000</t>
+          <t>08/12/1981</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
@@ -55856,7 +55856,7 @@
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>11-9081</t>
+          <t>29-2092</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
@@ -55866,7 +55866,7 @@
       </c>
       <c r="I25" s="14" t="inlineStr">
         <is>
-          <t>Lodging Managers</t>
+          <t>Hearing Aid Specialists</t>
         </is>
       </c>
       <c r="J25" s="14" t="inlineStr">
@@ -55876,7 +55876,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>06/12/2024</t>
+          <t>03/22/2018</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -55904,12 +55904,12 @@
       <c r="R25" s="14" t="n"/>
       <c r="S25" s="14" t="inlineStr">
         <is>
-          <t>$15.82</t>
+          <t>$16.39</t>
         </is>
       </c>
       <c r="T25" s="13" t="inlineStr">
         <is>
-          <t>$23.73</t>
+          <t>$24.59</t>
         </is>
       </c>
       <c r="U25" s="11" t="inlineStr">
@@ -55939,18 +55939,18 @@
       </c>
       <c r="Z25" s="11" t="inlineStr">
         <is>
-          <t>$34,300.00</t>
+          <t>$35,500.00</t>
         </is>
       </c>
       <c r="AA25" s="11" t="n"/>
       <c r="AB25" s="11" t="inlineStr">
         <is>
-          <t>$15.38</t>
+          <t>$15.91</t>
         </is>
       </c>
       <c r="AC25" s="11" t="inlineStr">
         <is>
-          <t>$23.07</t>
+          <t>$23.87</t>
         </is>
       </c>
       <c r="AD25" s="11" t="inlineStr">
@@ -55960,7 +55960,7 @@
       </c>
       <c r="AE25" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="AF25" s="11" t="inlineStr">
@@ -55970,18 +55970,18 @@
       </c>
       <c r="AG25" s="11" t="inlineStr">
         <is>
-          <t>$33,300.00</t>
+          <t>$34,500.00</t>
         </is>
       </c>
       <c r="AH25" s="11" t="n"/>
       <c r="AI25" s="11" t="inlineStr">
         <is>
-          <t>$14.90</t>
+          <t>$15.48</t>
         </is>
       </c>
       <c r="AJ25" s="11" t="inlineStr">
         <is>
-          <t>$22.35</t>
+          <t>$23.22</t>
         </is>
       </c>
       <c r="AK25" s="11" t="inlineStr">
@@ -56001,18 +56001,18 @@
       </c>
       <c r="AN25" s="11" t="inlineStr">
         <is>
-          <t>$32,300.00</t>
+          <t>$33,500.00</t>
         </is>
       </c>
       <c r="AO25" s="11" t="n"/>
       <c r="AP25" s="11" t="inlineStr">
         <is>
-          <t>$14.47</t>
+          <t>$15.00</t>
         </is>
       </c>
       <c r="AQ25" s="11" t="inlineStr">
         <is>
-          <t>$21.71</t>
+          <t>$22.50</t>
         </is>
       </c>
       <c r="AR25" s="11" t="inlineStr">
@@ -56032,7 +56032,7 @@
       </c>
       <c r="AU25" s="11" t="inlineStr">
         <is>
-          <t>$31,400.00</t>
+          <t>$32,500.00</t>
         </is>
       </c>
       <c r="AV25" s="11" t="inlineStr">
@@ -56100,7 +56100,7 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>08/08/1997</t>
+          <t>08/04/1977</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
@@ -56125,7 +56125,7 @@
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t>43-5061</t>
+          <t>15-1299</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
@@ -56135,7 +56135,7 @@
       </c>
       <c r="I26" s="14" t="inlineStr">
         <is>
-          <t>Production, Planning, and Expediting Clerks</t>
+          <t>Computer Occupations, All Other</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
@@ -56145,7 +56145,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>01/24/2022</t>
+          <t>07/16/2016</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56173,12 +56173,12 @@
       <c r="R26" s="14" t="n"/>
       <c r="S26" s="14" t="inlineStr">
         <is>
-          <t>$15.82</t>
+          <t>$20.53</t>
         </is>
       </c>
       <c r="T26" s="13" t="inlineStr">
         <is>
-          <t>$23.73</t>
+          <t>$30.80</t>
         </is>
       </c>
       <c r="U26" s="11" t="inlineStr">
@@ -56198,7 +56198,7 @@
       </c>
       <c r="X26" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,800.00</t>
         </is>
       </c>
       <c r="Y26" s="11" t="inlineStr">
@@ -56208,18 +56208,18 @@
       </c>
       <c r="Z26" s="11" t="inlineStr">
         <is>
-          <t>$34,300.00</t>
+          <t>$44,500.00</t>
         </is>
       </c>
       <c r="AA26" s="11" t="n"/>
       <c r="AB26" s="11" t="inlineStr">
         <is>
-          <t>$15.38</t>
+          <t>$19.95</t>
         </is>
       </c>
       <c r="AC26" s="11" t="inlineStr">
         <is>
-          <t>$23.07</t>
+          <t>$29.92</t>
         </is>
       </c>
       <c r="AD26" s="11" t="inlineStr">
@@ -56229,7 +56229,7 @@
       </c>
       <c r="AE26" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="AF26" s="11" t="inlineStr">
@@ -56239,18 +56239,18 @@
       </c>
       <c r="AG26" s="11" t="inlineStr">
         <is>
-          <t>$33,300.00</t>
+          <t>$43,200.00</t>
         </is>
       </c>
       <c r="AH26" s="11" t="n"/>
       <c r="AI26" s="11" t="inlineStr">
         <is>
-          <t>$14.90</t>
+          <t>$19.33</t>
         </is>
       </c>
       <c r="AJ26" s="11" t="inlineStr">
         <is>
-          <t>$22.35</t>
+          <t>$28.99</t>
         </is>
       </c>
       <c r="AK26" s="11" t="inlineStr">
@@ -56260,7 +56260,7 @@
       </c>
       <c r="AL26" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="AM26" s="11" t="inlineStr">
@@ -56270,18 +56270,18 @@
       </c>
       <c r="AN26" s="11" t="inlineStr">
         <is>
-          <t>$32,300.00</t>
+          <t>$41,900.00</t>
         </is>
       </c>
       <c r="AO26" s="11" t="n"/>
       <c r="AP26" s="11" t="inlineStr">
         <is>
-          <t>$14.47</t>
+          <t>$18.80</t>
         </is>
       </c>
       <c r="AQ26" s="11" t="inlineStr">
         <is>
-          <t>$21.71</t>
+          <t>$28.20</t>
         </is>
       </c>
       <c r="AR26" s="11" t="inlineStr">
@@ -56291,7 +56291,7 @@
       </c>
       <c r="AS26" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AT26" s="11" t="inlineStr">
@@ -56301,7 +56301,7 @@
       </c>
       <c r="AU26" s="11" t="inlineStr">
         <is>
-          <t>$31,400.00</t>
+          <t>$40,700.00</t>
         </is>
       </c>
       <c r="AV26" s="11" t="inlineStr">
@@ -56369,7 +56369,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>02/18/1979</t>
+          <t>02/06/1999</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
@@ -56394,7 +56394,7 @@
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>49-3042</t>
+          <t>47-2011</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
@@ -56404,7 +56404,7 @@
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>Mobile Heavy Equipment Mechanics, Except Engines</t>
+          <t>Boilermakers</t>
         </is>
       </c>
       <c r="J27" s="14" t="inlineStr">
@@ -56414,7 +56414,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>07/08/2013</t>
+          <t>02/28/2022</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56447,7 +56447,7 @@
       </c>
       <c r="T27" s="13" t="inlineStr">
         <is>
-          <t>$23.73</t>
+          <t>$29.79</t>
         </is>
       </c>
       <c r="U27" s="11" t="inlineStr">
@@ -56467,7 +56467,7 @@
       </c>
       <c r="X27" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="Y27" s="11" t="inlineStr">
@@ -56483,12 +56483,12 @@
       <c r="AA27" s="11" t="n"/>
       <c r="AB27" s="11" t="inlineStr">
         <is>
-          <t>$15.38</t>
+          <t>$19.23</t>
         </is>
       </c>
       <c r="AC27" s="11" t="inlineStr">
         <is>
-          <t>$23.07</t>
+          <t>$28.84</t>
         </is>
       </c>
       <c r="AD27" s="11" t="inlineStr">
@@ -56498,7 +56498,7 @@
       </c>
       <c r="AE27" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="AF27" s="11" t="inlineStr">
@@ -56508,18 +56508,18 @@
       </c>
       <c r="AG27" s="11" t="inlineStr">
         <is>
-          <t>$33,300.00</t>
+          <t>$41,700.00</t>
         </is>
       </c>
       <c r="AH27" s="11" t="n"/>
       <c r="AI27" s="11" t="inlineStr">
         <is>
-          <t>$14.90</t>
+          <t>$18.70</t>
         </is>
       </c>
       <c r="AJ27" s="11" t="inlineStr">
         <is>
-          <t>$22.35</t>
+          <t>$28.05</t>
         </is>
       </c>
       <c r="AK27" s="11" t="inlineStr">
@@ -56529,7 +56529,7 @@
       </c>
       <c r="AL27" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AM27" s="11" t="inlineStr">
@@ -56539,18 +56539,18 @@
       </c>
       <c r="AN27" s="11" t="inlineStr">
         <is>
-          <t>$32,300.00</t>
+          <t>$40,500.00</t>
         </is>
       </c>
       <c r="AO27" s="11" t="n"/>
       <c r="AP27" s="11" t="inlineStr">
         <is>
-          <t>$14.47</t>
+          <t>$18.12</t>
         </is>
       </c>
       <c r="AQ27" s="11" t="inlineStr">
         <is>
-          <t>$21.71</t>
+          <t>$27.18</t>
         </is>
       </c>
       <c r="AR27" s="11" t="inlineStr">
@@ -56560,7 +56560,7 @@
       </c>
       <c r="AS27" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AT27" s="11" t="inlineStr">
@@ -56570,7 +56570,7 @@
       </c>
       <c r="AU27" s="11" t="inlineStr">
         <is>
-          <t>$31,400.00</t>
+          <t>$39,300.00</t>
         </is>
       </c>
       <c r="AV27" s="11" t="inlineStr">
@@ -56638,7 +56638,7 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>10/18/1967</t>
+          <t>04/04/1989</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
@@ -56663,7 +56663,7 @@
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>53-7065</t>
+          <t>29-1229</t>
         </is>
       </c>
       <c r="H28" s="14" t="inlineStr">
@@ -56673,7 +56673,7 @@
       </c>
       <c r="I28" s="14" t="inlineStr">
         <is>
-          <t>Stockers and Order Fillers</t>
+          <t>Urologists</t>
         </is>
       </c>
       <c r="J28" s="14" t="inlineStr">
@@ -56683,7 +56683,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>05/28/2019</t>
+          <t>02/25/2014</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56711,12 +56711,12 @@
       <c r="R28" s="14" t="n"/>
       <c r="S28" s="14" t="inlineStr">
         <is>
-          <t>$11.44</t>
+          <t>$24.81</t>
         </is>
       </c>
       <c r="T28" s="13" t="inlineStr">
         <is>
-          <t>$17.16</t>
+          <t>$37.21</t>
         </is>
       </c>
       <c r="U28" s="11" t="inlineStr">
@@ -56736,7 +56736,7 @@
       </c>
       <c r="X28" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$2,200.00</t>
         </is>
       </c>
       <c r="Y28" s="11" t="inlineStr">
@@ -56746,18 +56746,18 @@
       </c>
       <c r="Z28" s="11" t="inlineStr">
         <is>
-          <t>$24,800.00</t>
+          <t>$53,800.00</t>
         </is>
       </c>
       <c r="AA28" s="11" t="n"/>
       <c r="AB28" s="11" t="inlineStr">
         <is>
-          <t>$11.11</t>
+          <t>$24.09</t>
         </is>
       </c>
       <c r="AC28" s="11" t="inlineStr">
         <is>
-          <t>$16.66</t>
+          <t>$36.13</t>
         </is>
       </c>
       <c r="AD28" s="11" t="inlineStr">
@@ -56767,7 +56767,7 @@
       </c>
       <c r="AE28" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$2,100.00</t>
         </is>
       </c>
       <c r="AF28" s="11" t="inlineStr">
@@ -56777,18 +56777,18 @@
       </c>
       <c r="AG28" s="11" t="inlineStr">
         <is>
-          <t>$24,100.00</t>
+          <t>$52,200.00</t>
         </is>
       </c>
       <c r="AH28" s="11" t="n"/>
       <c r="AI28" s="11" t="inlineStr">
         <is>
-          <t>$10.82</t>
+          <t>$23.41</t>
         </is>
       </c>
       <c r="AJ28" s="11" t="inlineStr">
         <is>
-          <t>$16.23</t>
+          <t>$35.12</t>
         </is>
       </c>
       <c r="AK28" s="11" t="inlineStr">
@@ -56798,7 +56798,7 @@
       </c>
       <c r="AL28" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$2,000.00</t>
         </is>
       </c>
       <c r="AM28" s="11" t="inlineStr">
@@ -56808,18 +56808,18 @@
       </c>
       <c r="AN28" s="11" t="inlineStr">
         <is>
-          <t>$23,400.00</t>
+          <t>$50,700.00</t>
         </is>
       </c>
       <c r="AO28" s="11" t="n"/>
       <c r="AP28" s="11" t="inlineStr">
         <is>
-          <t>$10.48</t>
+          <t>$22.69</t>
         </is>
       </c>
       <c r="AQ28" s="11" t="inlineStr">
         <is>
-          <t>$15.72</t>
+          <t>$34.04</t>
         </is>
       </c>
       <c r="AR28" s="11" t="inlineStr">
@@ -56829,7 +56829,7 @@
       </c>
       <c r="AS28" s="11" t="inlineStr">
         <is>
-          <t>$900.00</t>
+          <t>$2,000.00</t>
         </is>
       </c>
       <c r="AT28" s="11" t="inlineStr">
@@ -56839,7 +56839,7 @@
       </c>
       <c r="AU28" s="11" t="inlineStr">
         <is>
-          <t>$22,700.00</t>
+          <t>$49,200.00</t>
         </is>
       </c>
       <c r="AV28" s="11" t="inlineStr">
@@ -56907,7 +56907,7 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>12/04/1981</t>
+          <t>12/16/1973</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
@@ -56932,7 +56932,7 @@
       </c>
       <c r="G29" s="14" t="inlineStr">
         <is>
-          <t>31-2011</t>
+          <t>15-1299</t>
         </is>
       </c>
       <c r="H29" s="14" t="inlineStr">
@@ -56942,7 +56942,7 @@
       </c>
       <c r="I29" s="14" t="inlineStr">
         <is>
-          <t>Occupational Therapy Assistants</t>
+          <t>Information Security Engineers</t>
         </is>
       </c>
       <c r="J29" s="14" t="inlineStr">
@@ -56952,7 +56952,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>06/17/2019</t>
+          <t>05/27/2022</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -56980,12 +56980,12 @@
       <c r="R29" s="14" t="n"/>
       <c r="S29" s="14" t="inlineStr">
         <is>
-          <t>$17.69</t>
+          <t>$17.84</t>
         </is>
       </c>
       <c r="T29" s="13" t="inlineStr">
         <is>
-          <t>$26.54</t>
+          <t>$26.76</t>
         </is>
       </c>
       <c r="U29" s="11" t="inlineStr">
@@ -57015,18 +57015,18 @@
       </c>
       <c r="Z29" s="11" t="inlineStr">
         <is>
-          <t>$38,300.00</t>
+          <t>$38,600.00</t>
         </is>
       </c>
       <c r="AA29" s="11" t="n"/>
       <c r="AB29" s="11" t="inlineStr">
         <is>
-          <t>$17.16</t>
+          <t>$17.31</t>
         </is>
       </c>
       <c r="AC29" s="11" t="inlineStr">
         <is>
-          <t>$25.74</t>
+          <t>$25.96</t>
         </is>
       </c>
       <c r="AD29" s="11" t="inlineStr">
@@ -57046,18 +57046,18 @@
       </c>
       <c r="AG29" s="11" t="inlineStr">
         <is>
-          <t>$37,200.00</t>
+          <t>$37,500.00</t>
         </is>
       </c>
       <c r="AH29" s="11" t="n"/>
       <c r="AI29" s="11" t="inlineStr">
         <is>
-          <t>$16.68</t>
+          <t>$16.78</t>
         </is>
       </c>
       <c r="AJ29" s="11" t="inlineStr">
         <is>
-          <t>$25.02</t>
+          <t>$25.17</t>
         </is>
       </c>
       <c r="AK29" s="11" t="inlineStr">
@@ -57067,7 +57067,7 @@
       </c>
       <c r="AL29" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="AM29" s="11" t="inlineStr">
@@ -57077,18 +57077,18 @@
       </c>
       <c r="AN29" s="11" t="inlineStr">
         <is>
-          <t>$36,100.00</t>
+          <t>$36,400.00</t>
         </is>
       </c>
       <c r="AO29" s="11" t="n"/>
       <c r="AP29" s="11" t="inlineStr">
         <is>
-          <t>$16.15</t>
+          <t>$16.30</t>
         </is>
       </c>
       <c r="AQ29" s="11" t="inlineStr">
         <is>
-          <t>$24.22</t>
+          <t>$24.45</t>
         </is>
       </c>
       <c r="AR29" s="11" t="inlineStr">
@@ -57108,7 +57108,7 @@
       </c>
       <c r="AU29" s="11" t="inlineStr">
         <is>
-          <t>$35,000.00</t>
+          <t>$35,300.00</t>
         </is>
       </c>
       <c r="AV29" s="11" t="inlineStr">
@@ -57176,12 +57176,12 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>02/06/1991</t>
+          <t>09/01/1970</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -57201,7 +57201,7 @@
       </c>
       <c r="G30" s="14" t="inlineStr">
         <is>
-          <t>15-1299</t>
+          <t>31-9099</t>
         </is>
       </c>
       <c r="H30" s="14" t="inlineStr">
@@ -57211,7 +57211,7 @@
       </c>
       <c r="I30" s="14" t="inlineStr">
         <is>
-          <t>Information Technology Project Managers</t>
+          <t>Healthcare Support Workers, All Other</t>
         </is>
       </c>
       <c r="J30" s="14" t="inlineStr">
@@ -57221,7 +57221,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>02/25/2021</t>
+          <t>06/11/2022</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57249,12 +57249,12 @@
       <c r="R30" s="14" t="n"/>
       <c r="S30" s="14" t="inlineStr">
         <is>
-          <t>$19.09</t>
+          <t>$10.77</t>
         </is>
       </c>
       <c r="T30" s="13" t="inlineStr">
         <is>
-          <t>$28.63</t>
+          <t>$16.16</t>
         </is>
       </c>
       <c r="U30" s="11" t="inlineStr">
@@ -57274,7 +57274,7 @@
       </c>
       <c r="X30" s="11" t="inlineStr">
         <is>
-          <t>$1,700.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="Y30" s="11" t="inlineStr">
@@ -57284,18 +57284,18 @@
       </c>
       <c r="Z30" s="11" t="inlineStr">
         <is>
-          <t>$41,400.00</t>
+          <t>$23,300.00</t>
         </is>
       </c>
       <c r="AA30" s="11" t="n"/>
       <c r="AB30" s="11" t="inlineStr">
         <is>
-          <t>$18.56</t>
+          <t>$10.43</t>
         </is>
       </c>
       <c r="AC30" s="11" t="inlineStr">
         <is>
-          <t>$27.84</t>
+          <t>$15.64</t>
         </is>
       </c>
       <c r="AD30" s="11" t="inlineStr">
@@ -57305,7 +57305,7 @@
       </c>
       <c r="AE30" s="11" t="inlineStr">
         <is>
-          <t>$1,600.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="AF30" s="11" t="inlineStr">
@@ -57315,18 +57315,18 @@
       </c>
       <c r="AG30" s="11" t="inlineStr">
         <is>
-          <t>$40,200.00</t>
+          <t>$22,600.00</t>
         </is>
       </c>
       <c r="AH30" s="11" t="n"/>
       <c r="AI30" s="11" t="inlineStr">
         <is>
-          <t>$17.98</t>
+          <t>$10.10</t>
         </is>
       </c>
       <c r="AJ30" s="11" t="inlineStr">
         <is>
-          <t>$26.97</t>
+          <t>$15.15</t>
         </is>
       </c>
       <c r="AK30" s="11" t="inlineStr">
@@ -57336,7 +57336,7 @@
       </c>
       <c r="AL30" s="11" t="inlineStr">
         <is>
-          <t>$1,600.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="AM30" s="11" t="inlineStr">
@@ -57346,18 +57346,18 @@
       </c>
       <c r="AN30" s="11" t="inlineStr">
         <is>
-          <t>$39,000.00</t>
+          <t>$21,900.00</t>
         </is>
       </c>
       <c r="AO30" s="11" t="n"/>
       <c r="AP30" s="11" t="inlineStr">
         <is>
-          <t>$17.50</t>
+          <t>$9.81</t>
         </is>
       </c>
       <c r="AQ30" s="11" t="inlineStr">
         <is>
-          <t>$26.25</t>
+          <t>$14.71</t>
         </is>
       </c>
       <c r="AR30" s="11" t="inlineStr">
@@ -57367,7 +57367,7 @@
       </c>
       <c r="AS30" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$900.00</t>
         </is>
       </c>
       <c r="AT30" s="11" t="inlineStr">
@@ -57377,7 +57377,7 @@
       </c>
       <c r="AU30" s="11" t="inlineStr">
         <is>
-          <t>$37,900.00</t>
+          <t>$21,300.00</t>
         </is>
       </c>
       <c r="AV30" s="11" t="inlineStr">
@@ -57445,12 +57445,12 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>10/10/1999</t>
+          <t>07/07/1976</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -57470,7 +57470,7 @@
       </c>
       <c r="G31" s="14" t="inlineStr">
         <is>
-          <t>47-4011</t>
+          <t>51-2021</t>
         </is>
       </c>
       <c r="H31" s="14" t="inlineStr">
@@ -57480,7 +57480,7 @@
       </c>
       <c r="I31" s="14" t="inlineStr">
         <is>
-          <t>Energy Auditors</t>
+          <t>Coil Winders, Tapers, and Finishers</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
@@ -57490,7 +57490,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>06/25/2018</t>
+          <t>11/18/2025</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57518,12 +57518,12 @@
       <c r="R31" s="14" t="n"/>
       <c r="S31" s="14" t="inlineStr">
         <is>
-          <t>$22.84</t>
+          <t>$12.50</t>
         </is>
       </c>
       <c r="T31" s="13" t="inlineStr">
         <is>
-          <t>$34.26</t>
+          <t>$18.75</t>
         </is>
       </c>
       <c r="U31" s="11" t="inlineStr">
@@ -57543,7 +57543,7 @@
       </c>
       <c r="X31" s="11" t="inlineStr">
         <is>
-          <t>$2,000.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="Y31" s="11" t="inlineStr">
@@ -57553,18 +57553,18 @@
       </c>
       <c r="Z31" s="11" t="inlineStr">
         <is>
-          <t>$49,500.00</t>
+          <t>$27,100.00</t>
         </is>
       </c>
       <c r="AA31" s="11" t="n"/>
       <c r="AB31" s="11" t="inlineStr">
         <is>
-          <t>$22.21</t>
+          <t>$12.12</t>
         </is>
       </c>
       <c r="AC31" s="11" t="inlineStr">
         <is>
-          <t>$33.31</t>
+          <t>$18.18</t>
         </is>
       </c>
       <c r="AD31" s="11" t="inlineStr">
@@ -57574,7 +57574,7 @@
       </c>
       <c r="AE31" s="11" t="inlineStr">
         <is>
-          <t>$1,900.00</t>
+          <t>$1,100.00</t>
         </is>
       </c>
       <c r="AF31" s="11" t="inlineStr">
@@ -57584,18 +57584,18 @@
       </c>
       <c r="AG31" s="11" t="inlineStr">
         <is>
-          <t>$48,100.00</t>
+          <t>$26,300.00</t>
         </is>
       </c>
       <c r="AH31" s="11" t="n"/>
       <c r="AI31" s="11" t="inlineStr">
         <is>
-          <t>$21.54</t>
+          <t>$11.78</t>
         </is>
       </c>
       <c r="AJ31" s="11" t="inlineStr">
         <is>
-          <t>$32.31</t>
+          <t>$17.67</t>
         </is>
       </c>
       <c r="AK31" s="11" t="inlineStr">
@@ -57605,7 +57605,7 @@
       </c>
       <c r="AL31" s="11" t="inlineStr">
         <is>
-          <t>$1,900.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="AM31" s="11" t="inlineStr">
@@ -57615,18 +57615,18 @@
       </c>
       <c r="AN31" s="11" t="inlineStr">
         <is>
-          <t>$46,700.00</t>
+          <t>$25,500.00</t>
         </is>
       </c>
       <c r="AO31" s="11" t="n"/>
       <c r="AP31" s="11" t="inlineStr">
         <is>
-          <t>$20.91</t>
+          <t>$11.44</t>
         </is>
       </c>
       <c r="AQ31" s="11" t="inlineStr">
         <is>
-          <t>$31.37</t>
+          <t>$17.16</t>
         </is>
       </c>
       <c r="AR31" s="11" t="inlineStr">
@@ -57636,7 +57636,7 @@
       </c>
       <c r="AS31" s="11" t="inlineStr">
         <is>
-          <t>$1,800.00</t>
+          <t>$1,000.00</t>
         </is>
       </c>
       <c r="AT31" s="11" t="inlineStr">
@@ -57646,7 +57646,7 @@
       </c>
       <c r="AU31" s="11" t="inlineStr">
         <is>
-          <t>$45,300.00</t>
+          <t>$24,800.00</t>
         </is>
       </c>
       <c r="AV31" s="11" t="inlineStr">
@@ -57714,7 +57714,7 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>10/10/1979</t>
+          <t>06/10/1983</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
@@ -57739,7 +57739,7 @@
       </c>
       <c r="G32" s="14" t="inlineStr">
         <is>
-          <t>53-5031</t>
+          <t>29-1051</t>
         </is>
       </c>
       <c r="H32" s="14" t="inlineStr">
@@ -57749,7 +57749,7 @@
       </c>
       <c r="I32" s="14" t="inlineStr">
         <is>
-          <t>Ship Engineers</t>
+          <t>Pharmacists</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
@@ -57759,7 +57759,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>06/20/2023</t>
+          <t>01/01/2024</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57787,12 +57787,12 @@
       <c r="R32" s="14" t="n"/>
       <c r="S32" s="14" t="inlineStr">
         <is>
-          <t>$28.80</t>
+          <t>$32.16</t>
         </is>
       </c>
       <c r="T32" s="13" t="inlineStr">
         <is>
-          <t>$43.20</t>
+          <t>$48.24</t>
         </is>
       </c>
       <c r="U32" s="11" t="inlineStr">
@@ -57812,7 +57812,7 @@
       </c>
       <c r="X32" s="11" t="inlineStr">
         <is>
-          <t>$2,500.00</t>
+          <t>$2,800.00</t>
         </is>
       </c>
       <c r="Y32" s="11" t="inlineStr">
@@ -57822,18 +57822,18 @@
       </c>
       <c r="Z32" s="11" t="inlineStr">
         <is>
-          <t>$62,400.00</t>
+          <t>$69,700.00</t>
         </is>
       </c>
       <c r="AA32" s="11" t="n"/>
       <c r="AB32" s="11" t="inlineStr">
         <is>
-          <t>$27.98</t>
+          <t>$31.25</t>
         </is>
       </c>
       <c r="AC32" s="11" t="inlineStr">
         <is>
-          <t>$41.97</t>
+          <t>$46.88</t>
         </is>
       </c>
       <c r="AD32" s="11" t="inlineStr">
@@ -57843,7 +57843,7 @@
       </c>
       <c r="AE32" s="11" t="inlineStr">
         <is>
-          <t>$2,400.00</t>
+          <t>$2,700.00</t>
         </is>
       </c>
       <c r="AF32" s="11" t="inlineStr">
@@ -57853,18 +57853,18 @@
       </c>
       <c r="AG32" s="11" t="inlineStr">
         <is>
-          <t>$60,600.00</t>
+          <t>$67,700.00</t>
         </is>
       </c>
       <c r="AH32" s="11" t="n"/>
       <c r="AI32" s="11" t="inlineStr">
         <is>
-          <t>$27.12</t>
+          <t>$30.34</t>
         </is>
       </c>
       <c r="AJ32" s="11" t="inlineStr">
         <is>
-          <t>$40.68</t>
+          <t>$45.51</t>
         </is>
       </c>
       <c r="AK32" s="11" t="inlineStr">
@@ -57874,7 +57874,7 @@
       </c>
       <c r="AL32" s="11" t="inlineStr">
         <is>
-          <t>$2,400.00</t>
+          <t>$2,600.00</t>
         </is>
       </c>
       <c r="AM32" s="11" t="inlineStr">
@@ -57884,18 +57884,18 @@
       </c>
       <c r="AN32" s="11" t="inlineStr">
         <is>
-          <t>$58,800.00</t>
+          <t>$65,700.00</t>
         </is>
       </c>
       <c r="AO32" s="11" t="n"/>
       <c r="AP32" s="11" t="inlineStr">
         <is>
-          <t>$26.35</t>
+          <t>$29.42</t>
         </is>
       </c>
       <c r="AQ32" s="11" t="inlineStr">
         <is>
-          <t>$39.53</t>
+          <t>$44.13</t>
         </is>
       </c>
       <c r="AR32" s="11" t="inlineStr">
@@ -57905,7 +57905,7 @@
       </c>
       <c r="AS32" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$2,600.00</t>
         </is>
       </c>
       <c r="AT32" s="11" t="inlineStr">
@@ -57915,7 +57915,7 @@
       </c>
       <c r="AU32" s="11" t="inlineStr">
         <is>
-          <t>$57,100.00</t>
+          <t>$63,800.00</t>
         </is>
       </c>
       <c r="AV32" s="11" t="inlineStr">
@@ -57983,7 +57983,7 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>11/19/1992</t>
+          <t>07/23/1992</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>29-1124</t>
+          <t>19-4021</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -58018,7 +58018,7 @@
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>Radiation Therapists</t>
+          <t>Biological Technicians</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
@@ -58028,7 +58028,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>06/13/2020</t>
+          <t>07/10/2020</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58056,12 +58056,12 @@
       <c r="R33" s="14" t="n"/>
       <c r="S33" s="14" t="inlineStr">
         <is>
-          <t>$27.74</t>
+          <t>$14.57</t>
         </is>
       </c>
       <c r="T33" s="13" t="inlineStr">
         <is>
-          <t>$41.61</t>
+          <t>$21.86</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -58081,7 +58081,7 @@
       </c>
       <c r="X33" s="11" t="inlineStr">
         <is>
-          <t>$2,400.00</t>
+          <t>$1,300.00</t>
         </is>
       </c>
       <c r="Y33" s="11" t="inlineStr">
@@ -58091,18 +58091,18 @@
       </c>
       <c r="Z33" s="11" t="inlineStr">
         <is>
-          <t>$60,100.00</t>
+          <t>$31,600.00</t>
         </is>
       </c>
       <c r="AA33" s="11" t="n"/>
       <c r="AB33" s="11" t="inlineStr">
         <is>
-          <t>$26.92</t>
+          <t>$14.18</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>$40.38</t>
+          <t>$21.27</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
@@ -58112,7 +58112,7 @@
       </c>
       <c r="AE33" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$1,200.00</t>
         </is>
       </c>
       <c r="AF33" s="11" t="inlineStr">
@@ -58122,18 +58122,18 @@
       </c>
       <c r="AG33" s="11" t="inlineStr">
         <is>
-          <t>$58,300.00</t>
+          <t>$30,700.00</t>
         </is>
       </c>
       <c r="AH33" s="11" t="n"/>
       <c r="AI33" s="11" t="inlineStr">
         <is>
-          <t>$26.11</t>
+          <t>$13.75</t>
         </is>
       </c>
       <c r="AJ33" s="11" t="inlineStr">
         <is>
-          <t>$39.16</t>
+          <t>$20.62</t>
         </is>
       </c>
       <c r="AK33" s="11" t="inlineStr">
@@ -58143,7 +58143,7 @@
       </c>
       <c r="AL33" s="11" t="inlineStr">
         <is>
-          <t>$2,300.00</t>
+          <t>$1,200.00</t>
         </is>
       </c>
       <c r="AM33" s="11" t="inlineStr">
@@ -58153,18 +58153,18 @@
       </c>
       <c r="AN33" s="11" t="inlineStr">
         <is>
-          <t>$56,600.00</t>
+          <t>$29,800.00</t>
         </is>
       </c>
       <c r="AO33" s="11" t="n"/>
       <c r="AP33" s="11" t="inlineStr">
         <is>
-          <t>$25.38</t>
+          <t>$13.32</t>
         </is>
       </c>
       <c r="AQ33" s="11" t="inlineStr">
         <is>
-          <t>$38.07</t>
+          <t>$19.98</t>
         </is>
       </c>
       <c r="AR33" s="11" t="inlineStr">
@@ -58174,7 +58174,7 @@
       </c>
       <c r="AS33" s="11" t="inlineStr">
         <is>
-          <t>$2,200.00</t>
+          <t>$1,200.00</t>
         </is>
       </c>
       <c r="AT33" s="11" t="inlineStr">
@@ -58184,7 +58184,7 @@
       </c>
       <c r="AU33" s="11" t="inlineStr">
         <is>
-          <t>$55,000.00</t>
+          <t>$28,900.00</t>
         </is>
       </c>
       <c r="AV33" s="11" t="inlineStr">
@@ -58252,12 +58252,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>02/26/1971</t>
+          <t>01/09/1990</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
@@ -58277,7 +58277,7 @@
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>31-1132</t>
+          <t>19-3039</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
@@ -58287,7 +58287,7 @@
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>Orderlies</t>
+          <t>Clinical Neuropsychologists</t>
         </is>
       </c>
       <c r="J34" s="14" t="inlineStr">
@@ -58297,7 +58297,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>06/06/2013</t>
+          <t>10/21/2012</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58325,12 +58325,12 @@
       <c r="R34" s="14" t="n"/>
       <c r="S34" s="14" t="inlineStr">
         <is>
-          <t>$13.27</t>
+          <t>$17.55</t>
         </is>
       </c>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>$19.91</t>
+          <t>$26.33</t>
         </is>
       </c>
       <c r="U34" s="11" t="inlineStr">
@@ -58350,7 +58350,7 @@
       </c>
       <c r="X34" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="Y34" s="11" t="inlineStr">
@@ -58360,18 +58360,18 @@
       </c>
       <c r="Z34" s="11" t="inlineStr">
         <is>
-          <t>$28,800.00</t>
+          <t>$38,000.00</t>
         </is>
       </c>
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="11" t="inlineStr">
         <is>
-          <t>$12.93</t>
+          <t>$17.02</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>$19.39</t>
+          <t>$25.53</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
@@ -58381,7 +58381,7 @@
       </c>
       <c r="AE34" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="AF34" s="11" t="inlineStr">
@@ -58391,18 +58391,18 @@
       </c>
       <c r="AG34" s="11" t="inlineStr">
         <is>
-          <t>$28,000.00</t>
+          <t>$36,900.00</t>
         </is>
       </c>
       <c r="AH34" s="11" t="n"/>
       <c r="AI34" s="11" t="inlineStr">
         <is>
-          <t>$12.55</t>
+          <t>$16.54</t>
         </is>
       </c>
       <c r="AJ34" s="11" t="inlineStr">
         <is>
-          <t>$18.83</t>
+          <t>$24.81</t>
         </is>
       </c>
       <c r="AK34" s="11" t="inlineStr">
@@ -58412,7 +58412,7 @@
       </c>
       <c r="AL34" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="AM34" s="11" t="inlineStr">
@@ -58422,18 +58422,18 @@
       </c>
       <c r="AN34" s="11" t="inlineStr">
         <is>
-          <t>$27,200.00</t>
+          <t>$35,800.00</t>
         </is>
       </c>
       <c r="AO34" s="11" t="n"/>
       <c r="AP34" s="11" t="inlineStr">
         <is>
-          <t>$12.16</t>
+          <t>$16.06</t>
         </is>
       </c>
       <c r="AQ34" s="11" t="inlineStr">
         <is>
-          <t>$18.24</t>
+          <t>$24.09</t>
         </is>
       </c>
       <c r="AR34" s="11" t="inlineStr">
@@ -58443,7 +58443,7 @@
       </c>
       <c r="AS34" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$1,400.00</t>
         </is>
       </c>
       <c r="AT34" s="11" t="inlineStr">
@@ -58453,7 +58453,7 @@
       </c>
       <c r="AU34" s="11" t="inlineStr">
         <is>
-          <t>$26,400.00</t>
+          <t>$34,800.00</t>
         </is>
       </c>
       <c r="AV34" s="11" t="inlineStr">
@@ -58521,12 +58521,12 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>11/07/1996</t>
+          <t>08/20/1997</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
@@ -58546,7 +58546,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>51-9011</t>
+          <t>17-2121</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
@@ -58556,7 +58556,7 @@
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>Chemical Equipment Operators and Tenders</t>
+          <t>Marine Engineers and Naval Architects</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
@@ -58566,7 +58566,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>04/27/2022</t>
+          <t>02/03/2020</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -58594,12 +58594,12 @@
       <c r="R35" s="14" t="n"/>
       <c r="S35" s="14" t="inlineStr">
         <is>
-          <t>$13.22</t>
+          <t>$32.07</t>
         </is>
       </c>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>$19.83</t>
+          <t>$48.11</t>
         </is>
       </c>
       <c r="U35" s="11" t="inlineStr">
@@ -58619,7 +58619,7 @@
       </c>
       <c r="X35" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$2,800.00</t>
         </is>
       </c>
       <c r="Y35" s="11" t="inlineStr">
@@ -58629,18 +58629,18 @@
       </c>
       <c r="Z35" s="11" t="inlineStr">
         <is>
-          <t>$28,600.00</t>
+          <t>$69,500.00</t>
         </is>
       </c>
       <c r="AA35" s="11" t="n"/>
       <c r="AB35" s="11" t="inlineStr">
         <is>
-          <t>$12.84</t>
+          <t>$31.15</t>
         </is>
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>$19.26</t>
+          <t>$46.72</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
@@ -58650,7 +58650,7 @@
       </c>
       <c r="AE35" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$2,700.00</t>
         </is>
       </c>
       <c r="AF35" s="11" t="inlineStr">
@@ -58660,18 +58660,18 @@
       </c>
       <c r="AG35" s="11" t="inlineStr">
         <is>
-          <t>$27,800.00</t>
+          <t>$67,500.00</t>
         </is>
       </c>
       <c r="AH35" s="11" t="n"/>
       <c r="AI35" s="11" t="inlineStr">
         <is>
-          <t>$12.45</t>
+          <t>$30.24</t>
         </is>
       </c>
       <c r="AJ35" s="11" t="inlineStr">
         <is>
-          <t>$18.67</t>
+          <t>$45.36</t>
         </is>
       </c>
       <c r="AK35" s="11" t="inlineStr">
@@ -58681,7 +58681,7 @@
       </c>
       <c r="AL35" s="11" t="inlineStr">
         <is>
-          <t>$1,100.00</t>
+          <t>$2,600.00</t>
         </is>
       </c>
       <c r="AM35" s="11" t="inlineStr">
@@ -58691,18 +58691,18 @@
       </c>
       <c r="AN35" s="11" t="inlineStr">
         <is>
-          <t>$27,000.00</t>
+          <t>$65,500.00</t>
         </is>
       </c>
       <c r="AO35" s="11" t="n"/>
       <c r="AP35" s="11" t="inlineStr">
         <is>
-          <t>$12.12</t>
+          <t>$29.38</t>
         </is>
       </c>
       <c r="AQ35" s="11" t="inlineStr">
         <is>
-          <t>$18.18</t>
+          <t>$44.07</t>
         </is>
       </c>
       <c r="AR35" s="11" t="inlineStr">
@@ -58712,7 +58712,7 @@
       </c>
       <c r="AS35" s="11" t="inlineStr">
         <is>
-          <t>$1,000.00</t>
+          <t>$2,500.00</t>
         </is>
       </c>
       <c r="AT35" s="11" t="inlineStr">
@@ -58722,7 +58722,7 @@
       </c>
       <c r="AU35" s="11" t="inlineStr">
         <is>
-          <t>$26,200.00</t>
+          <t>$63,600.00</t>
         </is>
       </c>
       <c r="AV35" s="11" t="inlineStr">
@@ -65462,7 +65462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-20 19:47 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-21 18:05 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(data): E33 city-ordinance case, and re-sync the downloadable fixtures
Adds the edge case for an employee working inside a city paid-sick-leave
ordinance, which FF-010 showed the engine ignores. The description says
plainly that it is NOT applied today: the reference screen lists all 42
jurisdictions while the engine reads only the 25 state rows, so a
Berkeley employee is costed at 40 hours instead of 48 and the
remediation is understated.

edge_psl 6 -> 7 rows in the catalogue, and the downloadable workbook is
re-synced so the row is actually there.

Verified on a scratch Postgres 16: E33 lands in the Paid Sick Leave
group only, the Healthcare group is untouched, and the row count
updates.
</commit_message>
<xml_diff>
--- a/public/fixtures/all_combined.xlsx
+++ b/public/fixtures/all_combined.xlsx
@@ -53146,7 +53146,7 @@
       </c>
       <c r="B9" s="43" t="inlineStr">
         <is>
-          <t>07/21/2026</t>
+          <t>07/22/2026</t>
         </is>
       </c>
       <c r="C9" s="43" t="n"/>
@@ -53940,12 +53940,12 @@
       </c>
       <c r="B18" s="22" t="inlineStr">
         <is>
-          <t>08/12/1981</t>
+          <t>09/01/1970</t>
         </is>
       </c>
       <c r="C18" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D18" s="21" t="inlineStr">
@@ -53985,7 +53985,7 @@
       </c>
       <c r="K18" s="14" t="inlineStr">
         <is>
-          <t>03/04/2013</t>
+          <t>06/18/2013</t>
         </is>
       </c>
       <c r="L18" s="14" t="n"/>
@@ -54209,12 +54209,12 @@
       </c>
       <c r="B19" s="22" t="inlineStr">
         <is>
-          <t>12/12/1997</t>
+          <t>11/23/1988</t>
         </is>
       </c>
       <c r="C19" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
@@ -54254,7 +54254,7 @@
       </c>
       <c r="K19" s="14" t="inlineStr">
         <is>
-          <t>05/26/2021</t>
+          <t>03/10/2014</t>
         </is>
       </c>
       <c r="L19" s="14" t="n"/>
@@ -54478,12 +54478,12 @@
       </c>
       <c r="B20" s="22" t="inlineStr">
         <is>
-          <t>08/24/1985</t>
+          <t>03/07/1988</t>
         </is>
       </c>
       <c r="C20" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D20" s="21" t="inlineStr">
@@ -54523,7 +54523,7 @@
       </c>
       <c r="K20" s="14" t="inlineStr">
         <is>
-          <t>02/06/2019</t>
+          <t>12/25/2022</t>
         </is>
       </c>
       <c r="L20" s="14" t="n"/>
@@ -54763,12 +54763,12 @@
       </c>
       <c r="B21" s="22" t="inlineStr">
         <is>
-          <t>08/12/1997</t>
+          <t>07/27/1984</t>
         </is>
       </c>
       <c r="C21" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
@@ -54808,7 +54808,7 @@
       </c>
       <c r="K21" s="14" t="inlineStr">
         <is>
-          <t>03/03/2017</t>
+          <t>03/15/2019</t>
         </is>
       </c>
       <c r="L21" s="14" t="n"/>
@@ -55032,7 +55032,7 @@
       </c>
       <c r="B22" s="22" t="inlineStr">
         <is>
-          <t>12/04/1985</t>
+          <t>02/10/1971</t>
         </is>
       </c>
       <c r="C22" s="21" t="inlineStr">
@@ -55077,7 +55077,7 @@
       </c>
       <c r="K22" s="14" t="inlineStr">
         <is>
-          <t>06/10/2012</t>
+          <t>08/02/2024</t>
         </is>
       </c>
       <c r="L22" s="14" t="n"/>
@@ -55566,12 +55566,12 @@
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>11/19/2000</t>
+          <t>04/24/1981</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -55607,7 +55607,7 @@
       </c>
       <c r="K24" s="14" t="inlineStr">
         <is>
-          <t>09/06/2020</t>
+          <t>12/11/2019</t>
         </is>
       </c>
       <c r="L24" s="14" t="n"/>
@@ -55831,12 +55831,12 @@
       </c>
       <c r="B25" s="22" t="inlineStr">
         <is>
-          <t>08/12/1981</t>
+          <t>05/21/1970</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
@@ -55876,7 +55876,7 @@
       </c>
       <c r="K25" s="14" t="inlineStr">
         <is>
-          <t>03/22/2018</t>
+          <t>01/04/2025</t>
         </is>
       </c>
       <c r="L25" s="14" t="n"/>
@@ -56100,7 +56100,7 @@
       </c>
       <c r="B26" s="22" t="inlineStr">
         <is>
-          <t>08/04/1977</t>
+          <t>08/12/1977</t>
         </is>
       </c>
       <c r="C26" s="21" t="inlineStr">
@@ -56145,7 +56145,7 @@
       </c>
       <c r="K26" s="14" t="inlineStr">
         <is>
-          <t>07/16/2016</t>
+          <t>12/18/2015</t>
         </is>
       </c>
       <c r="L26" s="14" t="n"/>
@@ -56369,7 +56369,7 @@
       </c>
       <c r="B27" s="22" t="inlineStr">
         <is>
-          <t>02/06/1999</t>
+          <t>12/20/1985</t>
         </is>
       </c>
       <c r="C27" s="21" t="inlineStr">
@@ -56414,7 +56414,7 @@
       </c>
       <c r="K27" s="14" t="inlineStr">
         <is>
-          <t>02/28/2022</t>
+          <t>04/03/2015</t>
         </is>
       </c>
       <c r="L27" s="14" t="n"/>
@@ -56638,12 +56638,12 @@
       </c>
       <c r="B28" s="22" t="inlineStr">
         <is>
-          <t>04/04/1989</t>
+          <t>11/27/1976</t>
         </is>
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
@@ -56683,7 +56683,7 @@
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
-          <t>02/25/2014</t>
+          <t>08/05/2020</t>
         </is>
       </c>
       <c r="L28" s="14" t="n"/>
@@ -56907,12 +56907,12 @@
       </c>
       <c r="B29" s="22" t="inlineStr">
         <is>
-          <t>12/16/1973</t>
+          <t>09/13/1978</t>
         </is>
       </c>
       <c r="C29" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -56952,7 +56952,7 @@
       </c>
       <c r="K29" s="14" t="inlineStr">
         <is>
-          <t>05/27/2022</t>
+          <t>04/02/2025</t>
         </is>
       </c>
       <c r="L29" s="14" t="n"/>
@@ -57176,7 +57176,7 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
-          <t>09/01/1970</t>
+          <t>09/13/1962</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr">
@@ -57221,7 +57221,7 @@
       </c>
       <c r="K30" s="14" t="inlineStr">
         <is>
-          <t>06/11/2022</t>
+          <t>04/03/2019</t>
         </is>
       </c>
       <c r="L30" s="14" t="n"/>
@@ -57445,7 +57445,7 @@
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>07/07/1976</t>
+          <t>09/25/1978</t>
         </is>
       </c>
       <c r="C31" s="21" t="inlineStr">
@@ -57490,7 +57490,7 @@
       </c>
       <c r="K31" s="14" t="inlineStr">
         <is>
-          <t>11/18/2025</t>
+          <t>06/12/2012</t>
         </is>
       </c>
       <c r="L31" s="14" t="n"/>
@@ -57714,7 +57714,7 @@
       </c>
       <c r="B32" s="22" t="inlineStr">
         <is>
-          <t>06/10/1983</t>
+          <t>12/28/1981</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
@@ -57759,7 +57759,7 @@
       </c>
       <c r="K32" s="14" t="inlineStr">
         <is>
-          <t>01/01/2024</t>
+          <t>12/07/2019</t>
         </is>
       </c>
       <c r="L32" s="14" t="n"/>
@@ -57983,12 +57983,12 @@
       </c>
       <c r="B33" s="22" t="inlineStr">
         <is>
-          <t>07/23/1992</t>
+          <t>10/10/1991</t>
         </is>
       </c>
       <c r="C33" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D33" s="21" t="inlineStr">
@@ -58008,7 +58008,7 @@
       </c>
       <c r="G33" s="14" t="inlineStr">
         <is>
-          <t>19-4021</t>
+          <t>19-3051</t>
         </is>
       </c>
       <c r="H33" s="14" t="inlineStr">
@@ -58018,7 +58018,7 @@
       </c>
       <c r="I33" s="14" t="inlineStr">
         <is>
-          <t>Biological Technicians</t>
+          <t>Urban and Regional Planners</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
@@ -58028,7 +58028,7 @@
       </c>
       <c r="K33" s="14" t="inlineStr">
         <is>
-          <t>07/10/2020</t>
+          <t>03/18/2016</t>
         </is>
       </c>
       <c r="L33" s="14" t="n"/>
@@ -58056,12 +58056,12 @@
       <c r="R33" s="14" t="n"/>
       <c r="S33" s="14" t="inlineStr">
         <is>
-          <t>$14.57</t>
+          <t>$19.18</t>
         </is>
       </c>
       <c r="T33" s="13" t="inlineStr">
         <is>
-          <t>$21.86</t>
+          <t>$28.77</t>
         </is>
       </c>
       <c r="U33" s="11" t="inlineStr">
@@ -58081,7 +58081,7 @@
       </c>
       <c r="X33" s="11" t="inlineStr">
         <is>
-          <t>$1,300.00</t>
+          <t>$1,700.00</t>
         </is>
       </c>
       <c r="Y33" s="11" t="inlineStr">
@@ -58091,18 +58091,18 @@
       </c>
       <c r="Z33" s="11" t="inlineStr">
         <is>
-          <t>$31,600.00</t>
+          <t>$41,600.00</t>
         </is>
       </c>
       <c r="AA33" s="11" t="n"/>
       <c r="AB33" s="11" t="inlineStr">
         <is>
-          <t>$14.18</t>
+          <t>$18.65</t>
         </is>
       </c>
       <c r="AC33" s="11" t="inlineStr">
         <is>
-          <t>$21.27</t>
+          <t>$27.97</t>
         </is>
       </c>
       <c r="AD33" s="11" t="inlineStr">
@@ -58112,7 +58112,7 @@
       </c>
       <c r="AE33" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AF33" s="11" t="inlineStr">
@@ -58122,18 +58122,18 @@
       </c>
       <c r="AG33" s="11" t="inlineStr">
         <is>
-          <t>$30,700.00</t>
+          <t>$40,400.00</t>
         </is>
       </c>
       <c r="AH33" s="11" t="n"/>
       <c r="AI33" s="11" t="inlineStr">
         <is>
-          <t>$13.75</t>
+          <t>$18.08</t>
         </is>
       </c>
       <c r="AJ33" s="11" t="inlineStr">
         <is>
-          <t>$20.62</t>
+          <t>$27.12</t>
         </is>
       </c>
       <c r="AK33" s="11" t="inlineStr">
@@ -58143,7 +58143,7 @@
       </c>
       <c r="AL33" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,600.00</t>
         </is>
       </c>
       <c r="AM33" s="11" t="inlineStr">
@@ -58153,18 +58153,18 @@
       </c>
       <c r="AN33" s="11" t="inlineStr">
         <is>
-          <t>$29,800.00</t>
+          <t>$39,200.00</t>
         </is>
       </c>
       <c r="AO33" s="11" t="n"/>
       <c r="AP33" s="11" t="inlineStr">
         <is>
-          <t>$13.32</t>
+          <t>$17.60</t>
         </is>
       </c>
       <c r="AQ33" s="11" t="inlineStr">
         <is>
-          <t>$19.98</t>
+          <t>$26.40</t>
         </is>
       </c>
       <c r="AR33" s="11" t="inlineStr">
@@ -58174,7 +58174,7 @@
       </c>
       <c r="AS33" s="11" t="inlineStr">
         <is>
-          <t>$1,200.00</t>
+          <t>$1,500.00</t>
         </is>
       </c>
       <c r="AT33" s="11" t="inlineStr">
@@ -58184,7 +58184,7 @@
       </c>
       <c r="AU33" s="11" t="inlineStr">
         <is>
-          <t>$28,900.00</t>
+          <t>$38,100.00</t>
         </is>
       </c>
       <c r="AV33" s="11" t="inlineStr">
@@ -58252,12 +58252,12 @@
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>01/09/1990</t>
+          <t>10/02/1963</t>
         </is>
       </c>
       <c r="C34" s="21" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D34" s="21" t="inlineStr">
@@ -58277,7 +58277,7 @@
       </c>
       <c r="G34" s="14" t="inlineStr">
         <is>
-          <t>19-3039</t>
+          <t>17-2112</t>
         </is>
       </c>
       <c r="H34" s="14" t="inlineStr">
@@ -58287,7 +58287,7 @@
       </c>
       <c r="I34" s="14" t="inlineStr">
         <is>
-          <t>Clinical Neuropsychologists</t>
+          <t>Industrial Engineers</t>
         </is>
       </c>
       <c r="J34" s="14" t="inlineStr">
@@ -58297,7 +58297,7 @@
       </c>
       <c r="K34" s="14" t="inlineStr">
         <is>
-          <t>10/21/2012</t>
+          <t>04/16/2013</t>
         </is>
       </c>
       <c r="L34" s="14" t="n"/>
@@ -58325,12 +58325,12 @@
       <c r="R34" s="14" t="n"/>
       <c r="S34" s="14" t="inlineStr">
         <is>
-          <t>$17.55</t>
+          <t>$27.16</t>
         </is>
       </c>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>$26.33</t>
+          <t>$40.74</t>
         </is>
       </c>
       <c r="U34" s="11" t="inlineStr">
@@ -58350,7 +58350,7 @@
       </c>
       <c r="X34" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$2,400.00</t>
         </is>
       </c>
       <c r="Y34" s="11" t="inlineStr">
@@ -58360,18 +58360,18 @@
       </c>
       <c r="Z34" s="11" t="inlineStr">
         <is>
-          <t>$38,000.00</t>
+          <t>$58,900.00</t>
         </is>
       </c>
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="11" t="inlineStr">
         <is>
-          <t>$17.02</t>
+          <t>$26.39</t>
         </is>
       </c>
       <c r="AC34" s="11" t="inlineStr">
         <is>
-          <t>$25.53</t>
+          <t>$39.59</t>
         </is>
       </c>
       <c r="AD34" s="11" t="inlineStr">
@@ -58381,7 +58381,7 @@
       </c>
       <c r="AE34" s="11" t="inlineStr">
         <is>
-          <t>$1,500.00</t>
+          <t>$2,300.00</t>
         </is>
       </c>
       <c r="AF34" s="11" t="inlineStr">
@@ -58391,18 +58391,18 @@
       </c>
       <c r="AG34" s="11" t="inlineStr">
         <is>
-          <t>$36,900.00</t>
+          <t>$57,200.00</t>
         </is>
       </c>
       <c r="AH34" s="11" t="n"/>
       <c r="AI34" s="11" t="inlineStr">
         <is>
-          <t>$16.54</t>
+          <t>$25.62</t>
         </is>
       </c>
       <c r="AJ34" s="11" t="inlineStr">
         <is>
-          <t>$24.81</t>
+          <t>$38.43</t>
         </is>
       </c>
       <c r="AK34" s="11" t="inlineStr">
@@ -58412,7 +58412,7 @@
       </c>
       <c r="AL34" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$2,200.00</t>
         </is>
       </c>
       <c r="AM34" s="11" t="inlineStr">
@@ -58422,18 +58422,18 @@
       </c>
       <c r="AN34" s="11" t="inlineStr">
         <is>
-          <t>$35,800.00</t>
+          <t>$55,500.00</t>
         </is>
       </c>
       <c r="AO34" s="11" t="n"/>
       <c r="AP34" s="11" t="inlineStr">
         <is>
-          <t>$16.06</t>
+          <t>$24.86</t>
         </is>
       </c>
       <c r="AQ34" s="11" t="inlineStr">
         <is>
-          <t>$24.09</t>
+          <t>$37.29</t>
         </is>
       </c>
       <c r="AR34" s="11" t="inlineStr">
@@ -58443,7 +58443,7 @@
       </c>
       <c r="AS34" s="11" t="inlineStr">
         <is>
-          <t>$1,400.00</t>
+          <t>$2,200.00</t>
         </is>
       </c>
       <c r="AT34" s="11" t="inlineStr">
@@ -58453,7 +58453,7 @@
       </c>
       <c r="AU34" s="11" t="inlineStr">
         <is>
-          <t>$34,800.00</t>
+          <t>$53,900.00</t>
         </is>
       </c>
       <c r="AV34" s="11" t="inlineStr">
@@ -58521,12 +58521,12 @@
       </c>
       <c r="B35" s="22" t="inlineStr">
         <is>
-          <t>08/20/1997</t>
+          <t>07/11/1964</t>
         </is>
       </c>
       <c r="C35" s="21" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
@@ -58546,7 +58546,7 @@
       </c>
       <c r="G35" s="14" t="inlineStr">
         <is>
-          <t>17-2121</t>
+          <t>15-2041</t>
         </is>
       </c>
       <c r="H35" s="14" t="inlineStr">
@@ -58556,7 +58556,7 @@
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>Marine Engineers and Naval Architects</t>
+          <t>Statisticians</t>
         </is>
       </c>
       <c r="J35" s="14" t="inlineStr">
@@ -58566,7 +58566,7 @@
       </c>
       <c r="K35" s="14" t="inlineStr">
         <is>
-          <t>02/03/2020</t>
+          <t>02/04/2020</t>
         </is>
       </c>
       <c r="L35" s="14" t="n"/>
@@ -58594,12 +58594,12 @@
       <c r="R35" s="14" t="n"/>
       <c r="S35" s="14" t="inlineStr">
         <is>
-          <t>$32.07</t>
+          <t>$23.17</t>
         </is>
       </c>
       <c r="T35" s="13" t="inlineStr">
         <is>
-          <t>$48.11</t>
+          <t>$34.76</t>
         </is>
       </c>
       <c r="U35" s="11" t="inlineStr">
@@ -58619,7 +58619,7 @@
       </c>
       <c r="X35" s="11" t="inlineStr">
         <is>
-          <t>$2,800.00</t>
+          <t>$2,000.00</t>
         </is>
       </c>
       <c r="Y35" s="11" t="inlineStr">
@@ -58629,18 +58629,18 @@
       </c>
       <c r="Z35" s="11" t="inlineStr">
         <is>
-          <t>$69,500.00</t>
+          <t>$50,200.00</t>
         </is>
       </c>
       <c r="AA35" s="11" t="n"/>
       <c r="AB35" s="11" t="inlineStr">
         <is>
-          <t>$31.15</t>
+          <t>$22.50</t>
         </is>
       </c>
       <c r="AC35" s="11" t="inlineStr">
         <is>
-          <t>$46.72</t>
+          <t>$33.75</t>
         </is>
       </c>
       <c r="AD35" s="11" t="inlineStr">
@@ -58650,7 +58650,7 @@
       </c>
       <c r="AE35" s="11" t="inlineStr">
         <is>
-          <t>$2,700.00</t>
+          <t>$1,900.00</t>
         </is>
       </c>
       <c r="AF35" s="11" t="inlineStr">
@@ -58660,18 +58660,18 @@
       </c>
       <c r="AG35" s="11" t="inlineStr">
         <is>
-          <t>$67,500.00</t>
+          <t>$48,700.00</t>
         </is>
       </c>
       <c r="AH35" s="11" t="n"/>
       <c r="AI35" s="11" t="inlineStr">
         <is>
-          <t>$30.24</t>
+          <t>$21.83</t>
         </is>
       </c>
       <c r="AJ35" s="11" t="inlineStr">
         <is>
-          <t>$45.36</t>
+          <t>$32.74</t>
         </is>
       </c>
       <c r="AK35" s="11" t="inlineStr">
@@ -58681,7 +58681,7 @@
       </c>
       <c r="AL35" s="11" t="inlineStr">
         <is>
-          <t>$2,600.00</t>
+          <t>$1,900.00</t>
         </is>
       </c>
       <c r="AM35" s="11" t="inlineStr">
@@ -58691,18 +58691,18 @@
       </c>
       <c r="AN35" s="11" t="inlineStr">
         <is>
-          <t>$65,500.00</t>
+          <t>$47,300.00</t>
         </is>
       </c>
       <c r="AO35" s="11" t="n"/>
       <c r="AP35" s="11" t="inlineStr">
         <is>
-          <t>$29.38</t>
+          <t>$21.20</t>
         </is>
       </c>
       <c r="AQ35" s="11" t="inlineStr">
         <is>
-          <t>$44.07</t>
+          <t>$31.80</t>
         </is>
       </c>
       <c r="AR35" s="11" t="inlineStr">
@@ -58712,7 +58712,7 @@
       </c>
       <c r="AS35" s="11" t="inlineStr">
         <is>
-          <t>$2,500.00</t>
+          <t>$1,800.00</t>
         </is>
       </c>
       <c r="AT35" s="11" t="inlineStr">
@@ -58722,7 +58722,7 @@
       </c>
       <c r="AU35" s="11" t="inlineStr">
         <is>
-          <t>$63,600.00</t>
+          <t>$45,900.00</t>
         </is>
       </c>
       <c r="AV35" s="11" t="inlineStr">
@@ -65462,7 +65462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>generated 2026-07-21 18:05 from the reference warehouse (public.ext_*)</t>
+          <t>generated 2026-07-22 14:39 from the reference warehouse (public.ext_*)</t>
         </is>
       </c>
     </row>

</xml_diff>